<commit_message>
Add Batch 4 school scraping (SVA, Pratt, MICA, CCA, MassArt, BU, U Michigan)
Scrapes student rosters from 7 more schools, bringing the master workbook
to 19 tabs / 1,749 students. Notable fixes: MICA's nested-list parsing bug,
SVA's ambiguous name-list terminators, U Michigan's Cloudflare-protected
gallery pages (via crawl4ai), and several UNVERIFIED-flagged entries where
source pages had genuinely ambiguous name formatting.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -19,6 +19,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMU" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UW-Madison" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ohio State" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pratt" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BU" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SVA" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MICA" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCA" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MassArt" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="U Michigan Stamps" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$326</definedName>
@@ -33,6 +40,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UW-Madison'!$A$5:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Ohio State'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Pratt'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'BU'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'SVA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'MICA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CCA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'U Michigan Stamps'!$A$5:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -14313,6 +14327,720 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Pratt Institute 2026 'Pratt Shows' pages — MFA Thesis Parts 1-2, BFA Painting/Drawing/Sculpture/Printmaking (clean 'Exhibiting Artists' lists), and BFA/MFA Photography shows (names UNVERIFIED — source lists them as ambiguous &lt;br&gt;-separated chunks, see notes column)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.pratt.edu/events/pratt-shows-mfa-thesis-exhibition-part-1/ (and 23 corresponding pratt-shows-* discipline/photography pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Boston University College of Fine Arts — 2024 MFA Thesis 'Exhibiting Students by Program' page (Painting, Sculpture, Visual Narrative, Print Media &amp; Photography, Graphic Design)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.bu.edu/cfa/featured-work/mfa-thesis-2024/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: SVA Events &amp; Exhibitions search (2026-dated exhibitions with an 'Exhibiting artists include' / 'Artists include' description) — names only; these exhibitions may mix current students, alumni, faculty, and guest artists together, not confirmed to be current students only</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://sva.edu/events/search/type/Exhibition (22 paginated list pages, individual event pages fetched for all 2026-dated exhibitions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: MICA Grad Show 2026 — 'Participating students' per-program pages (14 MA/MFA programs), each with name and website/Instagram link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.mica.edu/events-exhibitions/annual-events-series/commencement/grad-show-2026/ (14 program subpages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: California College of the Arts newsroom article announcing the 2026 MFA Fine Arts Thesis Exhibition (names only; the actual event pages on portal.cca.edu are behind a student/staff login wall and were not used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.cca.edu/newsroom/cca-presents-the-2026-mfa-fine-arts-graduate-exhibitions/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: MassArt 2026 MFA Thesis Exhibition, Parts I &amp; II — 'FEATURED ARTISTS' lists with name + program (names only, no email/portfolio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://calendar.massart.edu/event/2026-mfa-thesis-exhibition-PARTI; https://calendar.massart.edu/event/2026-spring-mfa-thesis-exhibition-part-ii</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: U Michigan Stamps 2025 MFA Thesis Exhibition page (clean, dated) plus the Graduate and Undergraduate Research &amp; Creative Work gallery pages (mixed: some entries have a reliable name+year, many are UNVERIFIED 'Name: Artwork Title' entries with no year and unconfirmed name/title order — see notes column per row). Site is behind a Cloudflare JS challenge; fetched via crawl4ai headless browser, not a plain HTTP fetch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://stamps.umich.edu/events/2025-mfa-thesis-exhibition; https://stamps.umich.edu/research-creative-work/graduate-work-mfa; https://stamps.umich.edu/research-creative-work/undergraduate-work</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with Batch 4 additions
712 students with emails across RIT, Otis, MCAD, UW-Madison, Parsons, CMU
(unchanged count — no new schools this batch added emails, but source data
refreshed to match latest scrape).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -19,6 +19,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMU" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UW-Madison" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ohio State" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pratt" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BU" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SVA" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MICA" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCA" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MassArt" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="U Michigan Stamps" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$326</definedName>
@@ -33,6 +40,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UW-Madison'!$A$5:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Ohio State'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Pratt'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'BU'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'SVA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'MICA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CCA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'U Michigan Stamps'!$A$5:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -14313,6 +14327,720 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Pratt Institute 2026 'Pratt Shows' pages — MFA Thesis Parts 1-2, BFA Painting/Drawing/Sculpture/Printmaking (clean 'Exhibiting Artists' lists), and BFA/MFA Photography shows (names UNVERIFIED — source lists them as ambiguous &lt;br&gt;-separated chunks, see notes column)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.pratt.edu/events/pratt-shows-mfa-thesis-exhibition-part-1/ (and 23 corresponding pratt-shows-* discipline/photography pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Boston University College of Fine Arts — 2024 MFA Thesis 'Exhibiting Students by Program' page (Painting, Sculpture, Visual Narrative, Print Media &amp; Photography, Graphic Design)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.bu.edu/cfa/featured-work/mfa-thesis-2024/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: SVA Events &amp; Exhibitions search (2026-dated exhibitions with an 'Exhibiting artists include' / 'Artists include' description) — names only; these exhibitions may mix current students, alumni, faculty, and guest artists together, not confirmed to be current students only</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://sva.edu/events/search/type/Exhibition (22 paginated list pages, individual event pages fetched for all 2026-dated exhibitions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: MICA Grad Show 2026 — 'Participating students' per-program pages (14 MA/MFA programs), each with name and website/Instagram link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.mica.edu/events-exhibitions/annual-events-series/commencement/grad-show-2026/ (14 program subpages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: California College of the Arts newsroom article announcing the 2026 MFA Fine Arts Thesis Exhibition (names only; the actual event pages on portal.cca.edu are behind a student/staff login wall and were not used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.cca.edu/newsroom/cca-presents-the-2026-mfa-fine-arts-graduate-exhibitions/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: MassArt 2026 MFA Thesis Exhibition, Parts I &amp; II — 'FEATURED ARTISTS' lists with name + program (names only, no email/portfolio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://calendar.massart.edu/event/2026-mfa-thesis-exhibition-PARTI; https://calendar.massart.edu/event/2026-spring-mfa-thesis-exhibition-part-ii</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: U Michigan Stamps 2025 MFA Thesis Exhibition page (clean, dated) plus the Graduate and Undergraduate Research &amp; Creative Work gallery pages (mixed: some entries have a reliable name+year, many are UNVERIFIED 'Name: Artwork Title' entries with no year and unconfirmed name/title order — see notes column per row). Site is behind a Cloudflare JS challenge; fetched via crawl4ai headless browser, not a plain HTTP fetch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://stamps.umich.edu/events/2025-mfa-thesis-exhibition; https://stamps.umich.edu/research-creative-work/graduate-work-mfa; https://stamps.umich.edu/research-creative-work/undergraduate-work</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with Batch 5 additions
Still 712 students with emails (RIT, Otis, MCAD, UW-Madison, Parsons, CMU) —
CalArts/UCLA/Columbia added no new emails this batch, but the file is
refreshed to match the latest full scrape state.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -26,6 +26,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCA" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MassArt" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="U Michigan Stamps" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalArts" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UCLA" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columbia College Chicago" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$326</definedName>
@@ -47,6 +50,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CCA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'U Michigan Stamps'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'CalArts'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'UCLA'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Columbia College Chicago'!$A$5:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20115,6 +20121,312 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: CalArts 'High Pass' BFA Class of 2026 group exhibition page (names only; site requires crawl4ai due to cookie-consent/Cloudflare Turnstile blocking a plain fetch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://calarts.edu/high-pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: UCLA Department of Art — current Graduate Students directory by area of study (Ceramics, Interdisciplinary Studio, New Genres, Painting and Drawing, Photography, Sculpture), each linking to a personal portfolio/Instagram where available</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.art.ucla.edu/graduate-students</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Columbia College Chicago — 'Human Condition' 2026 BA/BFA Fine Art Exhibition page, Hokin Gallery and C33 Gallery exhibitor lists (names only). Note: 2 of 24 names have unusual letter-spacing in the source HTML itself (e.g. 'Faith H o g a n') — kept verbatim, flagged in notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://students.colum.edu/ssac/exhibition-archives/Manifest-Exhibitions/2026/human-condition-2026-babfa-in-fine-art-exhibition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with Batch 6 additions
Still 712 students with emails — Iowa/UW Art/BGSU added no new emails
(none of these sources publish student contact info), but the file is
refreshed to match the latest full scrape state (25 school tabs total).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -29,6 +29,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalArts" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UCLA" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columbia College Chicago" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iowa" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UW Art" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BGSU" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$I$326</definedName>
@@ -53,6 +56,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'CalArts'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'UCLA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Columbia College Chicago'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Iowa'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'UW Art'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20427,6 +20433,312 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: University of Iowa School of Art, Art History, and Design — MFA Virtual Exhibitions page (2024-2026 cohorts), each linking to a Matterport 3D exhibition tour rather than a personal portfolio site</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://art.uiowa.edu/events/mfa-virtual-exhibitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: University of Washington 2026 MFA + MDes Thesis Exhibition page (Henry Art Gallery) — names only; source does not map a specific discipline to each individual student</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: BGSU ScholarWorks — School of Art MA and MFA Graduate Exhibitions, Portfolios, and Theses repository, 2025 cohort (thesis title + author name; portfolio_url is the repository record, not a personal site)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://scholarworks.bgsu.edu/ms_art/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with BGSU discovery (Syed Fatmi)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -20643,7 +20643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -20722,6 +20722,49 @@
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Syed Fatmi</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>syedway.digital@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://syedway.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Thesis title: "OMNISYS"; email and portfolio found via web search (personal site syedway.com, confirmed via matching thesis title/LinkedIn)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 3 more BGSU emails
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -58,7 +58,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Columbia College Chicago'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Iowa'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'UW Art'!$A$5:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20643,7 +20643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -20768,13 +20768,142 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nick Felaris</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nickfelaris@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://scholarworks.bgsu.edu/ms_art/543</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Thesis title: "Nick Felaris Master of Fine Arts"; email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rachel Krieger</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rachelle@rachellekrieger.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.rachellekrieger.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Thesis title: "Rachel Krieger"; email and portfolio confirmed by user via rachellekrieger.com contact page</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kamrun Mim</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>kamrunmim.print@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://kamrunnahermim.wordpress.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BGSU</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Thesis title: "Kamrun Mim"; email and portfolio confirmed by user via kamrunnahermim.wordpress.com/about (bio/CV section)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I6"/>
+  <autoFilter ref="A5:I9"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 4 new MassArt emails
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -51,7 +51,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'SVA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'MICA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CCA'!$A$5:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'U Michigan Stamps'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'CalArts'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'UCLA'!$A$5:$I$6</definedName>
@@ -14855,7 +14855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14937,13 +14937,185 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Olivia Greenberg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>oliviadylan129@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.oliviadylanphotography.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>MassArt</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site oliviadylanphotography.com contact page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Anastasia Sierra</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>info@anastasiasierra.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.anastasiasierra.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MassArt</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site anastasiasierra.com/about)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Shailee Thakkar</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>shailee.v.thakkar@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Studio Arts</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.shaileethakkar.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>MassArt</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site shaileethakkar.com/aboutme footer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Antonio Bailey</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>antoniobaileylocal@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.antoniobailey.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MassArt</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site antoniobailey.com/about)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I6"/>
+  <autoFilter ref="A5:I9"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 3 new CMU emails
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -43,7 +43,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Temple-Tyler'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'VCU'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Yale'!$A$5:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UW-Madison'!$A$5:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Ohio State'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Pratt'!$A$5:$I$6</definedName>
@@ -13094,7 +13094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13284,23 +13284,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Morgan Shankweiler</t>
+          <t>Amber N. Ford</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>morganshankweiler@gmail.com</t>
+          <t>studio@ambernford.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MFA Studio Art (Second-Year MFA)</t>
+          <t>MFA Studio Art (First-Year MFA)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https:\/\/morganthomasshankweiler.com\/home.html</t>
+          <t>https://www.ambernford.com/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -13314,28 +13314,32 @@
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site ambernford.com/info)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Naomi Chambers</t>
+          <t>Morgan Shankweiler</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ncchambe@andrew.cmu.edu</t>
+          <t>morganshankweiler@gmail.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MFA Studio Art (Third-Year MFA)</t>
+          <t>MFA Studio Art (Second-Year MFA)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://art.cmu.edu/people/naomi-chambers/</t>
+          <t>https:\/\/morganthomasshankweiler.com\/home.html</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -13354,23 +13358,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aleena Akbar Khan</t>
+          <t>Sarah Al-Sarraj</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>aleenaakbar99@gmail.com</t>
+          <t>info.sarahalsarraj@gmail.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MFA Studio Art (Second-Year MFA)</t>
+          <t>MFA Studio Art (First-Year MFA)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https:\/\/aleenaakbarkhan.cargo.site\/</t>
+          <t>https:\/\/www.sarahalsarraj.com\/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -13384,17 +13388,21 @@
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site sarahalsarraj.com)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bulumko Mbete</t>
+          <t>Naomi Chambers</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bmbete@andrew.cmu.edu</t>
+          <t>ncchambe@andrew.cmu.edu</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -13405,7 +13413,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://art.cmu.edu/people/bulumko-mbete/</t>
+          <t>https://art.cmu.edu/people/naomi-chambers/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -13424,12 +13432,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ashley Ross</t>
+          <t>Aleena Akbar Khan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>info@ashleyaross.com</t>
+          <t>aleenaakbar99@gmail.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13440,7 +13448,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https:\/\/www.ashleyaross.com</t>
+          <t>https:\/\/aleenaakbarkhan.cargo.site\/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -13456,13 +13464,122 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bulumko Mbete</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bmbete@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (Third-Year MFA)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/bulumko-mbete/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ashley Ross</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>info@ashleyaross.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (Second-Year MFA)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https:\/\/www.ashleyaross.com</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Stefanie Zito</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>info@stefaniezito.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (First-Year MFA)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https:\/\/www.stefaniezito.com\/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site stefaniezito.com, listed as 'info[at]stefaniezito.com' anti-scrape format)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I13"/>
+  <autoFilter ref="A5:I16"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6:G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6:H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 5 new Temple/Tyler emails
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RISD'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otis'!$A$5:$I$227</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Parsons'!$A$5:$I$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Temple-Tyler'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Temple-Tyler'!$A$5:$I$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'VCU'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Yale'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$16</definedName>
@@ -31146,7 +31146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -31228,13 +31228,228 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Charles Jarboe</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>charles.jarboe@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Glass</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.charles-jarboe.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site charles-jarboe.com/bio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Amanda Crain-Freeland</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>amandancrain@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Sculpture</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.amandacrainfreeland.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site amandacrainfreeland.com CV page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rae Helms</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Raehelmsprint@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://raehelms.ink/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site raehelms.ink)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Francesca Lally</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>francescalally@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.francescalally.net/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site francescalally.net/ccvv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lilly Buttitta</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>lbuttittaart@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://lillybuttitta.com/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site lillybuttitta.com)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I6"/>
+  <autoFilter ref="A5:I10"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 24 more confirmed emails
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -40,10 +40,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RISD'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otis'!$A$5:$I$227</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Parsons'!$A$5:$I$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Temple-Tyler'!$A$5:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Temple-Tyler'!$A$5:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'VCU'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Yale'!$A$5:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UW-Madison'!$A$5:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Ohio State'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Pratt'!$A$5:$I$6</definedName>
@@ -51,13 +51,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'SVA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'MICA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CCA'!$A$5:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MassArt'!$A$5:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'U Michigan Stamps'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'CalArts'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'UCLA'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Columbia College Chicago'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Iowa'!$A$5:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'UW Art'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'UW Art'!$A$5:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13094,7 +13094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13214,23 +13214,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anne Chen</t>
+          <t>Walter Smits</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>anny.e.chen@gmail.com</t>
+          <t>smits.walt@gmail.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MFA Studio Art (Second-Year MFA)</t>
+          <t>MFA Studio Art (First-Year MFA)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://art.cmu.edu/people/anne-chen/</t>
+          <t>https:\/\/waltersmits.com</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -13244,17 +13244,21 @@
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (site was returning HTTP 503 on repeated fetch attempts by this tool)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Logan Larsen</t>
+          <t>Anne Chen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>logantlarsen98@gmail.com</t>
+          <t>anny.e.chen@gmail.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -13265,7 +13269,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https:\/\/www.loganlarsen.com</t>
+          <t>https://art.cmu.edu/people/anne-chen/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -13284,12 +13288,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Amber N. Ford</t>
+          <t>Yiying Wang</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>studio@ambernford.com</t>
+          <t>yiyingwang194@gmail.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13300,7 +13304,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.ambernford.com/</t>
+          <t>https:\/\/yiyingwang666.com\/lander</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -13316,19 +13320,19 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Email and portfolio found via web search (own site ambernford.com/info)</t>
+          <t>Email confirmed by user (site was unresolvable by this tool's fetcher)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Morgan Shankweiler</t>
+          <t>Logan Larsen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>morganshankweiler@gmail.com</t>
+          <t>logantlarsen98@gmail.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -13339,7 +13343,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https:\/\/morganthomasshankweiler.com\/home.html</t>
+          <t>https:\/\/www.loganlarsen.com</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -13358,12 +13362,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sarah Al-Sarraj</t>
+          <t>Amber N. Ford</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>info.sarahalsarraj@gmail.com</t>
+          <t>studio@ambernford.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -13374,7 +13378,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https:\/\/www.sarahalsarraj.com\/</t>
+          <t>https://www.ambernford.com/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -13390,30 +13394,30 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Email found via web search (own site sarahalsarraj.com)</t>
+          <t>Email and portfolio found via web search (own site ambernford.com/info)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naomi Chambers</t>
+          <t>Morgan Shankweiler</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ncchambe@andrew.cmu.edu</t>
+          <t>morganshankweiler@gmail.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MFA Studio Art (Third-Year MFA)</t>
+          <t>MFA Studio Art (Second-Year MFA)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://art.cmu.edu/people/naomi-chambers/</t>
+          <t>https:\/\/morganthomasshankweiler.com\/home.html</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -13432,23 +13436,23 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aleena Akbar Khan</t>
+          <t>Sarah Al-Sarraj</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>aleenaakbar99@gmail.com</t>
+          <t>info.sarahalsarraj@gmail.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MFA Studio Art (Second-Year MFA)</t>
+          <t>MFA Studio Art (First-Year MFA)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https:\/\/aleenaakbarkhan.cargo.site\/</t>
+          <t>https:\/\/www.sarahalsarraj.com\/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -13462,17 +13466,21 @@
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site sarahalsarraj.com)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Bulumko Mbete</t>
+          <t>Naomi Chambers</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bmbete@andrew.cmu.edu</t>
+          <t>ncchambe@andrew.cmu.edu</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13483,7 +13491,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://art.cmu.edu/people/bulumko-mbete/</t>
+          <t>https://art.cmu.edu/people/naomi-chambers/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -13502,12 +13510,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ashley Ross</t>
+          <t>Aleena Akbar Khan</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>info@ashleyaross.com</t>
+          <t>aleenaakbar99@gmail.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13518,7 +13526,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https:\/\/www.ashleyaross.com</t>
+          <t>https:\/\/aleenaakbarkhan.cargo.site\/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -13537,49 +13545,119 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stefanie Zito</t>
+          <t>Bulumko Mbete</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>info@stefaniezito.com</t>
+          <t>bmbete@andrew.cmu.edu</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MFA Studio Art (First-Year MFA)</t>
+          <t>MFA Studio Art (Third-Year MFA)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
+          <t>https://art.cmu.edu/people/bulumko-mbete/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ashley Ross</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>info@ashleyaross.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (Second-Year MFA)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https:\/\/www.ashleyaross.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Stefanie Zito</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>info@stefaniezito.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (First-Year MFA)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>https:\/\/www.stefaniezito.com\/</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>CMU</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
         <is>
           <t>Email found via web search (own site stefaniezito.com, listed as 'info[at]stefaniezito.com' anti-scrape format)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I16"/>
+  <autoFilter ref="A5:I18"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14972,7 +15050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15143,17 +15221,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shailee Thakkar</t>
+          <t>Lisa Spencer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>shailee.v.thakkar@gmail.com</t>
+          <t>lisaspencergallery@gmail.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MFA Studio Arts</t>
+          <t>MFA Photography</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -15163,7 +15241,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.shaileethakkar.com/</t>
+          <t>https://visura.co/lspencer/about</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -15179,24 +15257,24 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Email and portfolio found via web search (own site shaileethakkar.com/aboutme footer)</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Antonio Bailey</t>
+          <t>Shailee Thakkar</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>antoniobaileylocal@gmail.com</t>
+          <t>shailee.v.thakkar@gmail.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MFA Photography</t>
+          <t>MFA Studio Arts</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -15206,7 +15284,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.antoniobailey.com/</t>
+          <t>https://www.shaileethakkar.com/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -15222,17 +15300,103 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
+          <t>Email and portfolio found via web search (own site shaileethakkar.com/aboutme footer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Antonio Bailey</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>antoniobaileylocal@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.antoniobailey.com/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>MassArt</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>Email and portfolio found via web search (own site antoniobailey.com/about)</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Suzi Grossman</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Photo@suzigrossman.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.suzigrossman.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MassArt</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (different address than the earlier unverified search-summary guess)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I9"/>
+  <autoFilter ref="A5:I11"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6:G9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -20830,7 +20994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -20912,13 +21076,271 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Li-Yuan Chiou</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>lychiou@uw.edu</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (UW address)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Victoria Mackender</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>victoriaa961@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.vamack.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Email confirmed by user via vamack.com (manual check, DNS-unreachable by this tool)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oscar Pearson</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>o2thescar@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://oscarpearsonart.wixsite.com/studio</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Email confirmed by user. NOTE: a different, unrelated Oscar Pearson (California muralist/gallery artist) also shows up in search — not to be confused with this student</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Chave Pichardo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>chavepichardostudios@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://henryart.org/exhibitions/2026-university-of-washington-mfa-mdes-thesis-exhibition</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Andrew Roibal</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AndrewRoibalArt@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://art.washington.edu/people/andrew-roibal</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (also has UW address aroibal@uw.edu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ryan Walters</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RyanWaltersFilms@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA/MDes (UW Art — discipline not specified per student)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.ryanwalters.art/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Email confirmed by user via ryanwalters.art (manual check, .art domain unreachable by this tool)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I6"/>
+  <autoFilter ref="A5:I11"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -31146,7 +31568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -31274,17 +31696,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Amanda Crain-Freeland</t>
+          <t>Natalia Purchiaroni</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>amandancrain@gmail.com</t>
+          <t>npurchphotography@gmail.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MFA Sculpture</t>
+          <t>MFA Photography</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -31292,11 +31714,7 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://www.amandacrainfreeland.com/</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -31310,24 +31728,24 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Email and portfolio found via web search (own site amandacrainfreeland.com CV page)</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rae Helms</t>
+          <t>Macy West</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Raehelmsprint@gmail.com</t>
+          <t>macywest99@gmail.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MFA Printmaking</t>
+          <t>MFA Fine Arts</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -31335,11 +31753,7 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://raehelms.ink/</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Temple/Tyler</t>
@@ -31353,24 +31767,24 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Email and portfolio found via web search (own site raehelms.ink)</t>
+          <t>Email confirmed by user</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Francesca Lally</t>
+          <t>Amanda Crain-Freeland</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>francescalally@gmail.com</t>
+          <t>amandancrain@gmail.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MFA Printmaking</t>
+          <t>MFA Sculpture</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -31380,7 +31794,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.francescalally.net/</t>
+          <t>https://www.amandacrainfreeland.com/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -31396,24 +31810,24 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Email and portfolio found via web search (own site francescalally.net/ccvv)</t>
+          <t>Email and portfolio found via web search (own site amandacrainfreeland.com CV page)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lilly Buttitta</t>
+          <t>Mika Obayashi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>lbuttittaart@gmail.com</t>
+          <t>mikacobayashi@gmail.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MFA Painting</t>
+          <t>MFA Fiber/Sculpture</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -31423,7 +31837,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://lillybuttitta.com/</t>
+          <t>https://www.mikaobayashi.com/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -31439,17 +31853,763 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Heather Swenson</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mail@heatherswenson.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.heatherswenson.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (own site heatherswenson.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sophia Dell'Arciprete</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sophiadellarciprete@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA Photography</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://sophiadellarciprete.com/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rae Helms</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Raehelmsprint@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://raehelms.ink/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site raehelms.ink)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Francesca Lally</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>francescalally@gmail.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MFA Printmaking</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://www.francescalally.net/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Email and portfolio found via web search (own site francescalally.net/ccvv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ari Zuaro</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>azuaro@theclaystudio.org</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MFA Ceramics</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://arizuaro.com/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (Clay Studio staff address, where they also work)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lilly Buttitta</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>lbuttittaart@gmail.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://lillybuttitta.com/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>Email and portfolio found via web search (own site lillybuttitta.com)</t>
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Esther Park</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>eyparkart7@gmail.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mollie Hansen</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>mollie.hansen.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Maedeh Mehdipour</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>mehdipour.maede@gmail.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MFA Fiber and Material Studies</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://maedehmehdipour.com/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (site was returning HTTP 403 on fetch by this tool)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Madeline Rodriguez</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>rodriguez.maddie@gmail.com</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ivy Jewell</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ijewell@theclaystudio.org</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (Clay Studio staff address)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Angelique Scott</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ArtByAngeliqueScott@gmail.com</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ben Solo</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>benweidlich.bs@gmail.com</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.bensoloart.com/</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (real name appears to be Ben Weidlich; site was unresolvable by this tool's fetcher)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Logan Crompton</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>lcrompton@kcai.edu</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://scoby.page/log3y-logan-crompton</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (Kansas City Art Institute address)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Boi Boy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>boiboy.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (full name may be 'Boi Boy Cottrell' per one source)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Diego Juarez</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>juarezcdiego@gmail.com</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.diegojuarez.com/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Gianna Santucci</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>gsantucci630@gmail.com</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Email confirmed by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Pegah Saebi</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pegah.saebi96@gmail.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MFA Design</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://pegahsaebi.com/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Temple/Tyler</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (site was unresolvable by this tool's fetcher)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I10"/>
+  <autoFilter ref="A5:I28"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6:G10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 6 new VCU emails
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -42,7 +42,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Otis'!$A$5:$I$227</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Parsons'!$A$5:$I$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Temple-Tyler'!$A$5:$I$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'VCU'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'VCU'!$A$5:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Yale'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UW-Madison'!$A$5:$I$24</definedName>
@@ -42516,7 +42516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -42598,13 +42598,271 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aya Khalife</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>khalifehaya7@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.ayakhalife.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Email confirmed by user (portfolio site ayakhalife.com, JS-rendered Readymag site, personal email surfaced via 'Reach out' mailto link only visible on hover — not captured by automated fetch/crawl4ai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rebecca Oh</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>rebeccaohart@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Painting and Printmaking</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>http://www.rebeccaoh.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site rebeccaoh.com/about, verified in raw HTML: 'Feel free to e-mail the artist at rebeccaohart@gmail.com')</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>David Guarnizo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>guarnizode@vcu.edu</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Photography and Film</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://arts.vcu.edu/directory/david-guarnizo/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Email found via web search (VCU School of the Arts directory page, verified in raw HTML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tyna Ontko</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ontkotyna@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Sculpture and Extended Media</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://tynaontko.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site tynaontko.com/contact, address was obfuscated as 'ontkotyna(at)gmail(dot)com' in page text, deobfuscated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Molly Garrett</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>hi@mollygarrett.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Graphic Design</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://mollygarrett.com/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site mollygarrett.com/contact, address was obfuscated as 'hi [at] mollygarrett.com' in page text, deobfuscated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Amy Duval</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>amys.duval@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Craft/Material Studies</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.duvalceramics.ca/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>VCU</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site duvalceramics.ca/contact, JS-rendered — found via interactive Playwright probe of the contact form page)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I6"/>
+  <autoFilter ref="A5:I11"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx with 4 new Ohio State emails
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -46,7 +46,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Yale'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMU'!$A$5:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UW-Madison'!$A$5:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Ohio State'!$A$5:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Ohio State'!$A$5:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Pratt'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'BU'!$A$5:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'SVA'!$A$5:$I$6</definedName>
@@ -14440,7 +14440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14522,13 +14522,185 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mandy Darrington</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>mandylynndarrington@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.mandydarrington.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ohio State</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site mandydarrington.com/about, obfuscated as 'mandylynndarrington [at] gmail [dot] com', deobfuscated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>William Evans</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>evans_william@live.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.williamevans.studio/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Ohio State</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site williamevans.studio/about, plain text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Andrew Mehall</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mehall.11@osu.edu</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://art.osu.edu/people/mehall.11</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ohio State</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Email found via web search (OSU Department of Art directory profile, institutional address, verified in raw HTML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ivan David Ng</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>info@ivandavidng.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Drawing and Painting</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.ivandavidng.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Ohio State</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Email found via web search (own site ivandavidng.com/about, plain text)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I6"/>
+  <autoFilter ref="A5:I9"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx: 5 new schools added (no new emails)
Mirrors main@2e21cac -- adds Alfred University, Cornell, UT Austin, Cooper
Union, and SCAD sheets (498 names, all currently email-less), completing
the original 28-school target list. No change to actual email count since
none of these 5 schools publish contact info on their source pages.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -34,6 +34,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BGSU" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalArts Animation" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAL Central Saint Martins" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alfred University" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UT Austin" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cooper Union" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCAD" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIT'!$A$5:$J$326</definedName>
@@ -63,6 +68,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'CalArts Animation'!$A$5:$J$256</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'UAL Central Saint Martins'!$A$5:$J$288</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Alfred University'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Cornell'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'UT Austin'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Cooper Union'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'SCAD'!$A$5:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -14323,7 +14333,11 @@
           <t>Name corrected from 'Anna!' (UW-Madison directory listed only a first name + exclamation point) to 'Anna Colombia', confirmed via her linked personal site (annacolombia.com) and Instagram (@anna.colombia). Email found via web search, verified in raw HTML mailto: link on annacolombia.com/contact</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15115,7 +15129,11 @@
           <t>Email found via web search (own site mandydarrington.com/about, obfuscated as 'mandylynndarrington [at] gmail [dot] com', deobfuscated)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15159,7 +15177,11 @@
           <t>Email confirmed by user via web search ('Annelise Duque artist email'). Not found in original pass despite checking her own site directly — the address itself doesn't appear to be published on annelise-duque.com's CV/contact pages, so likely surfaced from a different indexed source</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15203,7 +15225,11 @@
           <t>Email found via web search (own site williamevans.studio/about, plain text)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -15247,7 +15273,11 @@
           <t>Email confirmed by user via web search ('Josiah Jamison artist email'). OSU student email address, not found on his personal site (josiahjamison.com) which only had Squarespace placeholder text</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15291,7 +15321,11 @@
           <t>Email found via web search (OSU Department of Art directory profile, institutional address, verified in raw HTML)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -15335,7 +15369,11 @@
           <t>Email confirmed by user. OSU directory page (naylor.135) 404s on direct fetch as of 2026-08-15 despite surfacing in search results with this address — could not independently verify job title/current-student status the way Mehall's page allowed; used per user confirmation</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -15379,7 +15417,11 @@
           <t>Email found via web search (own site ivandavidng.com/about, plain text)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -15423,7 +15465,11 @@
           <t>Email confirmed by user. OSU directory page (robbins.391) 404s on direct fetch as of 2026-08-15 despite surfacing in search results with this address — could not independently verify job title/current-student status the way Mehall's page allowed; used per user confirmation</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -15467,7 +15513,11 @@
           <t>Email confirmed by user. OSU directory page (saraceni.4) 404s on direct fetch as of 2026-08-15 despite surfacing in search results with this address — could not independently verify job title/current-student status the way Mehall's page allowed; used per user confirmation</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15511,7 +15561,11 @@
           <t>Email confirmed by user. OSU directory page (trippe.5) 404s on direct fetch as of 2026-08-15 despite surfacing in search results with this address — could not independently verify job title/current-student status the way Mehall's page allowed; used per user confirmation</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15555,7 +15609,11 @@
           <t>Email confirmed by user via web search ('James Waite artist email'). Not found in original pass — no personal site had surfaced then either</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15599,7 +15657,11 @@
           <t>NAME CORRECTED from 'Shaheen Banerjee' — user independently confirmed via web search that the OSU directory has 'Shaheen Beardsley' (cartoonist), not 'Shaheen Banerjee'. Re-reading the raw source string ('Banerjee, Shaheen Beardsley, Maria Conlon, Onni Estabrook, Samuel Lo, Takahiro Okubo, Shruti Shankar, Sam Wrigglesworth, Xuan') confirms this: it's actually a plain 'Firstname Lastname, Firstname Lastname, ...' list, not the shifted 'Lastname, Firstname Lastname' pattern originally assumed — 'Shaheen' pairs with 'Beardsley' directly, not with the orphaned leading 'Banerjee' fragment. Email confirmed by user, OSU directory address</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15643,7 +15705,11 @@
           <t>NAME CORRECTED from 'Onni Conlon' — same re-reading as Beardsley above: 'Maria' pairs with 'Conlon' directly. Email confirmed by user, OSU directory address</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15687,7 +15753,11 @@
           <t>NAME CORRECTED from 'Samuel Estabrook' — same re-reading: 'Onni' pairs with 'Estabrook' directly. Email confirmed by user, OSU directory address. CAUTION: an earlier session found an OSU directory profile for an 'Onni Estabrook' bio'd as a Lecturer with a BFA from a different school — worth double-checking this isn't the same faculty-vs-student mix-up seen with Matthew Machado, though the user independently confirmed this address as correct for our 2026 MFA student</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15731,7 +15801,11 @@
           <t>NAME CORRECTED from 'Takahiro Lo' — same re-reading: 'Samuel' pairs with 'Lo' directly. Email confirmed by user (OSU student address; also has a general contact samuelloarts@gmail.com and a personal website per user's research, not yet added here)</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15775,7 +15849,11 @@
           <t>NAME CORRECTED from 'Shruti Okubo' — same re-reading: 'Takahiro' pairs with 'Okubo' directly. Email confirmed by user, OSU directory address</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:J21"/>
@@ -16467,7 +16545,11 @@
           <t>Email confirmed by user (business email for his 'Snailpirate' animator/artist persona)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -23107,7 +23189,11 @@
           <t>Email found via web search citing her UW Art + Art History + Design directory profile page (art.washington.edu/people/dahae-cheon), which 404s on a direct unauthenticated fetch — same unverifiable-but-plausible pattern as several Ohio State directory rows; used per user confirmation</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -23247,7 +23333,11 @@
           <t>Email found via web search citing her UW Art + Art History + Design directory profile page (art.washington.edu/people/alex-moni-sauri), which 404s on a direct unauthenticated fetch — same unverifiable-but-plausible pattern as several Ohio State directory rows; also has an active Instagram (@a.moni.sauri) confirming she's a current UW grad student; used per user confirmation</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -35039,7 +35129,11 @@
           <t>Medium: Sculpture; project 'CANG'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -35079,7 +35173,11 @@
           <t>Medium: Fiber and Material Arts; project 'Awaara (Strays)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -35119,7 +35217,11 @@
           <t>Medium: Painting/Drawing; project 'The Assembly: Portals I-VII'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -35159,7 +35261,11 @@
           <t>Medium: Photography; project 'Follow the Imaginary Line'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -35199,7 +35305,11 @@
           <t>Medium: Painting/Drawing; project 'Dreams of Inertion: The Discovery of a Parallel World, and the Portal in Croydon That led me There.'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -35239,7 +35349,11 @@
           <t>Medium: Painting/Drawing; project 'Commercial Break'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -35279,7 +35393,11 @@
           <t>Medium: Painting/Drawing; project ''ILoveMyComputer''; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -35319,7 +35437,11 @@
           <t>Medium: Design; project 'An Afrofuturist Manifesto'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -35359,7 +35481,11 @@
           <t>Medium: Design; project 'a.p.e - assimilation, preservation, evolution'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -35399,7 +35525,11 @@
           <t>Medium: Fiber and Material Arts; project 'Fanm de Faye'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -35439,7 +35569,11 @@
           <t>Medium: Painting/Drawing; project 'The Work of Men's Hands Guided by Their Brains'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -35479,7 +35613,11 @@
           <t>Medium: Painting/Drawing; project 'A Taste of Home'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -35519,7 +35657,11 @@
           <t>Medium: Sculpture; project 'To Y: Stationary Magpie Dream'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -35559,7 +35701,11 @@
           <t>Medium: Fashion; project 'ROMANIAN ROOTS'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -35599,7 +35745,11 @@
           <t>Medium: Design; project 'Cassandra'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -35639,7 +35789,11 @@
           <t>Medium: Painting/Drawing; project 'Patterns of a Life - Transforming Personal Data Into Human Stories'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -35679,7 +35833,11 @@
           <t>Medium: Fashion; project 'The Finite in the Infinite'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -35719,7 +35877,11 @@
           <t>Medium: Design; project 'Fathom - A Framework For Autonomous Cleansing'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -35759,7 +35921,11 @@
           <t>Medium: Painting/Drawing; project 'Texture of Dream'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -35799,7 +35965,11 @@
           <t>Medium: Painting/Drawing; project 'Chequered Lines'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -35839,7 +36009,11 @@
           <t>Medium: Painting/Drawing; project 'Working Hard, Hardly Working'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -35879,7 +36053,11 @@
           <t>Medium: Painting/Drawing; project 'Landing'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -35919,7 +36097,11 @@
           <t>Medium: Fiber and Material Arts; project 'Return to Earth'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -35959,7 +36141,11 @@
           <t>Medium: Painting/Drawing; project 'You Can't Park There Mate'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -35999,7 +36185,11 @@
           <t>Medium: 2D/3D Animation; project 'Did You Catch a Hare?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -36039,7 +36229,11 @@
           <t>Medium: Design; project 'Hannah and Piggy Try British(ish) Foods'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -36079,7 +36273,11 @@
           <t>Medium: Design; project 'LEADHER'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -36119,7 +36317,11 @@
           <t>Medium: Photography; project 'The Invisible Hotel: Capturing Photoplasm'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -36159,7 +36361,11 @@
           <t>Medium: Design; project 'Stay in your Lane'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -36199,7 +36405,11 @@
           <t>Medium: Sculpture; project 'American Burnout'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -36239,7 +36449,11 @@
           <t>Medium: Design; project 'Where Ideas Grow'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -36279,7 +36493,11 @@
           <t>Medium: Painting/Drawing; project 'On Waking Whilst Sleeping'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -36319,7 +36537,11 @@
           <t>Medium: Fiber and Material Arts; project 'Preservation grants permenance'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -36359,7 +36581,11 @@
           <t>Medium: Painting/Drawing; project 'Timekeeper's Toy'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -36399,7 +36625,11 @@
           <t>Medium: Fashion; project 'Portrait of the American Dream: Pre-Collection'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -36439,7 +36669,11 @@
           <t>Medium: Painting/Drawing; project 'Bitter Herbs'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -36479,7 +36713,11 @@
           <t>Medium: Fashion; project 'The Grim Reaper'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -36519,7 +36757,11 @@
           <t>Medium: Painting/Drawing; project 'A New Place to Drown'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -36559,7 +36801,11 @@
           <t>Medium: Painting/Drawing; project 'a dam for your eyes, is a constellation for me.'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -36599,7 +36845,11 @@
           <t>Medium: Painting/Drawing; project 'Capturing Contingency: The Paradoxical Connection Between Moving Image and Contingency'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -36639,7 +36889,11 @@
           <t>Medium: Fashion; project '''PINK MATRIX'''; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -36679,7 +36933,11 @@
           <t>Medium: Design; project 'lips, pfffrrrt - indignation'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -36719,7 +36977,11 @@
           <t>Medium: Fashion; project 'Editorial Design'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -36759,7 +37021,11 @@
           <t>Medium: Sculpture; project 'Hollow(core) Bench'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -36799,7 +37065,11 @@
           <t>Medium: Fiber and Material Arts; project 'Girlhood Across Generations'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -36839,7 +37109,11 @@
           <t>Medium: Design; project 'The Design EcoSystem'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -36879,7 +37153,11 @@
           <t>Medium: Design; project ''STATE''; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -36919,7 +37197,11 @@
           <t>Medium: Painting/Drawing; project 'Cyborg Botany'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -36959,7 +37241,11 @@
           <t>Medium: Fiber and Material Arts; project 'A Series of Totemic Objects'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -36999,7 +37285,11 @@
           <t>Medium: Painting/Drawing; project 'Mavourneen in {consumer}land'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -37039,7 +37329,11 @@
           <t>Medium: 2D/3D Animation; project 'SAM AND THE ENTITIES (2026)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -37079,7 +37373,11 @@
           <t>Medium: Painting/Drawing; project 'Permission To Touch - I Am What I Lived Through.'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -37119,7 +37417,11 @@
           <t>Medium: 2D/3D Animation; project 'Showreel 2026'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -37159,7 +37461,11 @@
           <t>Medium: Design; project 'NOVA'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -37199,7 +37505,11 @@
           <t>Medium: Painting/Drawing; project 'technofossils000'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -37239,7 +37549,11 @@
           <t>Medium: Photography; project 'Silence'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -37279,7 +37593,11 @@
           <t>Medium: Fiber and Material Arts; project 'Carrying System'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -37319,7 +37637,11 @@
           <t>Medium: Photography; project 'The Audience'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -37359,7 +37681,11 @@
           <t>Medium: Design; project 'An Illusion That Heals'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -37399,7 +37725,11 @@
           <t>Medium: Design; project 'Foreign Objects'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -37439,7 +37769,11 @@
           <t>Medium: Fiber and Material Arts; project 'When Sweetness Breaks'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -37479,7 +37813,11 @@
           <t>Medium: Photography; project 'Techniques of Hidden Coitus'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -37519,7 +37857,11 @@
           <t>Medium: Design; project 'Shinryeong Market'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -37559,7 +37901,11 @@
           <t>Medium: Painting/Drawing; project 'Lesbianism / Articulate'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -37599,7 +37945,11 @@
           <t>Medium: Design; project 'Designing with Nature: A Graphic Toolkit'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -37639,7 +37989,11 @@
           <t>Medium: Painting/Drawing; project 'Talking Statues'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -37679,7 +38033,11 @@
           <t>Medium: Design; project 'Who am I?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -37719,7 +38077,11 @@
           <t>Medium: Fiber and Material Arts; project 'Gemstones'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -37759,7 +38121,11 @@
           <t>Medium: Painting/Drawing; project 'Blood Stained Pass'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -37799,7 +38165,11 @@
           <t>Medium: Design; project 'IN BETWEEN: On Existing Between Languages'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -37839,7 +38209,11 @@
           <t>Medium: Design; project 'Chinese Internet Slang'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -37879,7 +38253,11 @@
           <t>Medium: Design; project 'SIDEKICK'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -37919,7 +38297,11 @@
           <t>Medium: Painting/Drawing; project 'Egg Fired Rice'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -37959,7 +38341,11 @@
           <t>Medium: Sculpture; project 'Interior Edges'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -37999,7 +38385,11 @@
           <t>Medium: Design; project 'Black Through Waves'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -38039,7 +38429,11 @@
           <t>Medium: Sculpture; project 'Soft Landscape'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -38079,7 +38473,11 @@
           <t>Medium: Fiber and Material Arts; project 'CHANGES'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -38119,7 +38517,11 @@
           <t>Medium: Design; project 'DUNYA (دنيا)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -38159,7 +38561,11 @@
           <t>Medium: Painting/Drawing; project 'In Pursuit of Muscle'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -38199,7 +38605,11 @@
           <t>Medium: Fiber and Material Arts; project 'Petrichor /the smell of rain/'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -38239,7 +38649,11 @@
           <t>Medium: Fiber and Material Arts; project 'The Gilded Lily'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -38279,7 +38693,11 @@
           <t>Medium: Fiber and Material Arts; project '15,000 Ft'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -38319,7 +38737,11 @@
           <t>Medium: Design; project 'The Unquiet Page'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -38359,7 +38781,11 @@
           <t>Medium: Design; project 'Milieu'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -38399,7 +38825,11 @@
           <t>Medium: Design; project 'The Grammar of Evidence'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -38439,7 +38869,11 @@
           <t>Medium: Design; project 'Please Press Play'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -38479,7 +38913,11 @@
           <t>Medium: Sculpture; project 'Loop'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -38519,7 +38957,11 @@
           <t>Medium: Photography; project 'The Sensortype'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -38559,7 +39001,11 @@
           <t>Medium: Fiber and Material Arts; project 'Traces of Pressure'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -38599,7 +39045,11 @@
           <t>Medium: Sculpture; project 'Maybe Pearl'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr"/>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -38639,7 +39089,11 @@
           <t>Medium: Design; project 'Report/Re-port/Port'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -38679,7 +39133,11 @@
           <t>Medium: Fashion; project 'Crafted Stories'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr"/>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -38719,7 +39177,11 @@
           <t>Medium: Design; project 'After the Look'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -38759,7 +39221,11 @@
           <t>Medium: Design; project 'Mingwei Zhang'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -38799,7 +39265,11 @@
           <t>Medium: Painting/Drawing; project '"Millennia"'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -38839,7 +39309,11 @@
           <t>Medium: Sculpture; project 'Ęhi - My Spiritual Guardians'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -38879,7 +39353,11 @@
           <t>Medium: Design; project 'The Vegas Paradox' (collaborative/group project — profile URL resolved to the project cover page, not a personal profile; name recovered from page &lt;title&gt; tag 'The Vegas Paradox - Rose Kessler - UAL Showcase'); email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -38919,7 +39397,11 @@
           <t>Medium: Painting/Drawing; project 'A Journey Without Love or Youth'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -38959,7 +39441,11 @@
           <t>Medium: Fiber and Material Arts; project 'surprise'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -38999,7 +39485,11 @@
           <t>Medium: Sculpture; project 'Dormiente - While we are asleep'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -39039,7 +39529,11 @@
           <t>Medium: Fiber and Material Arts; project 'Our Archive'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -39079,7 +39573,11 @@
           <t>Medium: Painting/Drawing; project 'Safety Yellow'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -39119,7 +39617,11 @@
           <t>Medium: Design; project 'After Revision… What Remains?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -39159,7 +39661,11 @@
           <t>Medium: Sculpture; project 'Modern Locus'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -39199,7 +39705,11 @@
           <t>Medium: Sculpture; project 'Ex-millinery'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr"/>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -39239,7 +39749,11 @@
           <t>Medium: Design; project 'A Publication for Different Ways of Thinking'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -39279,7 +39793,11 @@
           <t>Medium: Sculpture; project 'Something in Nothing'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -39319,7 +39837,11 @@
           <t>Medium: Design; project 'YAZ Magazine on Tatar Language Loss and Tactile Alphabet Set'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -39359,7 +39881,11 @@
           <t>Medium: Sculpture; project 'GROUND'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr"/>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -39399,7 +39925,11 @@
           <t>Medium: Design; project 'M3WD'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -39439,7 +39969,11 @@
           <t>Medium: Painting/Drawing; project 'The Spectacle'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr"/>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -39479,7 +40013,11 @@
           <t>Medium: Sculpture; project 'Dust 2 Dust'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -39519,7 +40057,11 @@
           <t>Medium: Painting/Drawing; project 'Sowing Seeds'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr"/>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -39559,7 +40101,11 @@
           <t>Medium: Sculpture; project 'Strand'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr"/>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -39599,7 +40145,11 @@
           <t>Medium: Filmmaking; project 'Walking With The Other Self'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -39639,7 +40189,11 @@
           <t>Medium: Fashion; project 'Aurora, Texas'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -39679,7 +40233,11 @@
           <t>Medium: Photography; project 'Between Illusion and Reality'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -39719,7 +40277,11 @@
           <t>Medium: Sculpture; project 'Mechanical Flowers'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -39759,7 +40321,11 @@
           <t>Medium: Design; project '#Bigben'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -39799,7 +40365,11 @@
           <t>Medium: Design; project 'When Poets Talk About Food'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -39839,7 +40409,11 @@
           <t>Medium: Design; project 'X( )Y( )Z( )'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr"/>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -39879,7 +40453,11 @@
           <t>Medium: Design; project 'Hearth'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -39919,7 +40497,11 @@
           <t>Medium: Fiber and Material Arts; project 'Eternity and a Day'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr"/>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -39959,7 +40541,11 @@
           <t>Medium: Design; project 'Creatives in the Wild'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -39999,7 +40585,11 @@
           <t>Medium: Sculpture; project 'LINII'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -40039,7 +40629,11 @@
           <t>Medium: Fiber and Material Arts; project 'Emotional Guardian'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -40079,7 +40673,11 @@
           <t>Medium: Painting/Drawing; project 'A Return'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr"/>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -40119,7 +40717,11 @@
           <t>Medium: Sculpture; project 'SPIRAL MOTION'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr"/>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -40159,7 +40761,11 @@
           <t>Medium: Design; project 'Margaret Killed Feminist Noise'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -40199,7 +40805,11 @@
           <t>Medium: Design; project 'Perform Again'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -40239,7 +40849,11 @@
           <t>Medium: Painting/Drawing; project 'Repleating'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -40279,7 +40893,11 @@
           <t>Medium: Design; project 'Removed From Circulation'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -40319,7 +40937,11 @@
           <t>Medium: Sculpture; project 'Traces'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -40359,7 +40981,11 @@
           <t>Medium: Sculpture; project 'Chimera Obscura'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr"/>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -40399,7 +41025,11 @@
           <t>Medium: Fiber and Material Arts; project 'Reframing The Invisible'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr"/>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -40439,7 +41069,11 @@
           <t>Medium: Fiber and Material Arts; project 'Militarisation of the Everyday'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -40479,7 +41113,11 @@
           <t>Medium: Photography; project 'My Dream is a Four-Square-Meter Large'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr"/>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -40519,7 +41157,11 @@
           <t>Medium: Painting/Drawing; project 'Between Here'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -40559,7 +41201,11 @@
           <t>Medium: Design; project 'Central Bureau of Geographic Cartography'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr"/>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -40599,7 +41245,11 @@
           <t>Medium: Sculpture; project 'Radience Core'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -40639,7 +41289,11 @@
           <t>Medium: Design; project 'Have You Ever Felt an Earthquake That Wasn't There?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -40679,7 +41333,11 @@
           <t>Medium: Fiber and Material Arts; project 'If I Were a Toy Bunny'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr"/>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -40719,7 +41377,11 @@
           <t>Medium: Fiber and Material Arts; project 'The Lost Sea Wand'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -40759,7 +41421,11 @@
           <t>Medium: Painting/Drawing; project 'From My Mouth'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -40799,7 +41465,11 @@
           <t>Medium: Sculpture; project 'S l o w  C e r a m i c'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -40839,7 +41509,11 @@
           <t>Medium: Design; project 'Home Is Where The...'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -40879,7 +41553,11 @@
           <t>Medium: Design; project 'The Last Generation of Pepper Farmers'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -40919,7 +41597,11 @@
           <t>Medium: Design; project 'Letter Variations: Text, Score, Voice'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -40959,7 +41641,11 @@
           <t>Medium: Design; project 'Decision Paralysis Atlas'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -40999,7 +41685,11 @@
           <t>Medium: Design; project 'Roots'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -41039,7 +41729,11 @@
           <t>Medium: 2D/3D Animation; project 'Suuugar!'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr"/>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -41079,7 +41773,11 @@
           <t>Medium: Design; project 'Red, White, and Who?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr"/>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -41119,7 +41817,11 @@
           <t>Medium: Design; project 'HIVE'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr"/>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -41159,7 +41861,11 @@
           <t>Medium: 2D/3D Animation; project 'Somewhere, Once'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -41199,7 +41905,11 @@
           <t>Medium: Design; project 'Rhythm of Body - Interactive Game That Arouses Your Bodily Awareness'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J160" t="inlineStr"/>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -41239,7 +41949,11 @@
           <t>Medium: Fiber and Material Arts; project 'Methods. Mechanisms. Materiality.'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -41279,7 +41993,11 @@
           <t>Medium: Sculpture; project 'Translated'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J162" t="inlineStr"/>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -41319,7 +42037,11 @@
           <t>Medium: Painting/Drawing; project 'Dear Moon,'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr"/>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -41359,7 +42081,11 @@
           <t>Medium: Painting/Drawing; project 'DoomScroll'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr"/>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -41399,7 +42125,11 @@
           <t>Medium: Sculpture; project 'Unintended'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -41439,7 +42169,11 @@
           <t>Medium: Design; project 'Dyslexia Strengths Kit'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J166" t="inlineStr"/>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -41479,7 +42213,11 @@
           <t>Medium: Design; project 'Smells in Layers'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -41519,7 +42257,11 @@
           <t>Medium: Design; project 'Unfolding Reading'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J168" t="inlineStr"/>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -41559,7 +42301,11 @@
           <t>Medium: Design; project 'How to use a Phone Using Your Body'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J169" t="inlineStr"/>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -41599,7 +42345,11 @@
           <t>Medium: Design; project 'Patterns Of Presence: Shared Presence in the Digital Age'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -41639,7 +42389,11 @@
           <t>Medium: Sculpture; project 'Industrial Jadeite Relics'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -41679,7 +42433,11 @@
           <t>Medium: Sculpture; project 'GAMETOPIA'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J172" t="inlineStr"/>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -41719,7 +42477,11 @@
           <t>Medium: Sculpture; project 'If Looks Could Kill'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J173" t="inlineStr"/>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -41759,7 +42521,11 @@
           <t>Medium: Design; project 'HYDE PARK AUDITORY MAP'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr"/>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -41799,7 +42565,11 @@
           <t>Medium: Fashion; project 'The Dishwashing Monologue: Lingering Whispers'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr"/>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -41839,7 +42609,11 @@
           <t>Medium: Fiber and Material Arts; project 'Ornament and Artifice'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J176" t="inlineStr"/>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -41879,7 +42653,11 @@
           <t>Medium: Painting/Drawing; project 'Rhizomatic Becoming in Deep Time'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -41919,7 +42697,11 @@
           <t>Medium: Painting/Drawing; project 'Doll-Like Sensibility'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J178" t="inlineStr"/>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -41959,7 +42741,11 @@
           <t>Medium: 2D/3D Animation; project 'What Do Your Parents Beat You With?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J179" t="inlineStr"/>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -41999,7 +42785,11 @@
           <t>Medium: Design; project 'Meaning as Gesture'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -42039,7 +42829,11 @@
           <t>Medium: 2D/3D Animation; project 'This Place is not a Place of Honour'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J181" t="inlineStr"/>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -42079,7 +42873,11 @@
           <t>Medium: Design; project 'Soma: Carried Across'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J182" t="inlineStr"/>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -42119,7 +42917,11 @@
           <t>Medium: Sculpture; project 'Emotive Enamel'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J183" t="inlineStr"/>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -42159,7 +42961,11 @@
           <t>Medium: Design; project 'Beyond Us'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J184" t="inlineStr"/>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -42199,7 +43005,11 @@
           <t>Medium: Design; project 'Requiem of the Potato'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J185" t="inlineStr"/>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -42239,7 +43049,11 @@
           <t>Medium: Sculpture; project 'Tales from the Table'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -42279,7 +43093,11 @@
           <t>Medium: Fiber and Material Arts; project 'Residual Logic'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr"/>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -42319,7 +43137,11 @@
           <t>Medium: Fiber and Material Arts; project 'Through a Frosted Window'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr"/>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -42359,7 +43181,11 @@
           <t>Medium: Fiber and Material Arts; project 'Entanglement'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -42399,7 +43225,11 @@
           <t>Medium: Filmmaking; project 'Light Leaks: Material Traces as Thresholds'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J190" t="inlineStr"/>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -42439,7 +43269,11 @@
           <t>Medium: Design; project 'Abyss'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J191" t="inlineStr"/>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -42479,7 +43313,11 @@
           <t>Medium: Design; project 'The Departure of Them, The Return of Us'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr"/>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -42519,7 +43357,11 @@
           <t>Medium: Sculpture; project 'A Really Soft Thing'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J193" t="inlineStr"/>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -42559,7 +43401,11 @@
           <t>Medium: Photography; project 'A Rose Is A Rose Is A Rose Is A Rose'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J194" t="inlineStr"/>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -42599,7 +43445,11 @@
           <t>Medium: Design; project 'Glory to the Irrelevant'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J195" t="inlineStr"/>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -42639,7 +43489,11 @@
           <t>Medium: Design; project 'JEONG'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J196" t="inlineStr"/>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -42679,7 +43533,11 @@
           <t>Medium: Sculpture; project ''Table Manners''; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J197" t="inlineStr"/>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -42719,7 +43577,11 @@
           <t>Medium: Fiber and Material Arts; project 'Textile Tender'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J198" t="inlineStr"/>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -42759,7 +43621,11 @@
           <t>Medium: Fiber and Material Arts; project 'Repertoire'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J199" t="inlineStr"/>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -42799,7 +43665,11 @@
           <t>Medium: Fiber and Material Arts; project 'Concluded Fragments'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -42839,7 +43709,11 @@
           <t>Medium: Design; project 'A Park in Time'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J201" t="inlineStr"/>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -42879,7 +43753,11 @@
           <t>Medium: 2D/3D Animation; project 'Chilli Chong Carne'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J202" t="inlineStr"/>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -42919,7 +43797,11 @@
           <t>Medium: Design; project 'Afterimage'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J203" t="inlineStr"/>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -42959,7 +43841,11 @@
           <t>Medium: 2D/3D Animation; project 'Felt Me'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -42999,7 +43885,11 @@
           <t>Medium: Painting/Drawing; project 'Creeping'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J205" t="inlineStr"/>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -43039,7 +43929,11 @@
           <t>Medium: Design; project 'What if all of Your Belongings had to fit Within one Carry-on Suitcase?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J206" t="inlineStr"/>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -43079,7 +43973,11 @@
           <t>Medium: Painting/Drawing; project 'Untitled World'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J207" t="inlineStr"/>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -43119,7 +44017,11 @@
           <t>Medium: Design; project 'Attunement'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -43159,7 +44061,11 @@
           <t>Medium: Painting/Drawing; project 'Bicce Monstrum (Accumulation and Sloughing)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -43199,7 +44105,11 @@
           <t>Medium: Design; project 'Where Did They Go?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr"/>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -43239,7 +44149,11 @@
           <t>Medium: Painting/Drawing; project 'LifeSpan'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J211" t="inlineStr"/>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -43279,7 +44193,11 @@
           <t>Medium: Fashion; project 'All We Ever Wanted Was Everything'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J212" t="inlineStr"/>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -43319,7 +44237,11 @@
           <t>Medium: Fashion; project 'I ran away from home, but where can I run away from longing?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J213" t="inlineStr"/>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -43359,7 +44281,11 @@
           <t>Medium: Painting/Drawing; project 'Unclocking Time'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J214" t="inlineStr"/>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -43399,7 +44325,11 @@
           <t>Medium: Painting/Drawing; project 'And Where Now?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J215" t="inlineStr"/>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -43439,7 +44369,11 @@
           <t>Medium: Design; project 'Bewnans Ort Mor (Life at Sea)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -43479,7 +44413,11 @@
           <t>Medium: Design; project 'Loneliness in Everyday Life'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J217" t="inlineStr"/>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -43519,7 +44457,11 @@
           <t>Medium: Design; project 'A Touch of Sin (Livestocks' Version)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J218" t="inlineStr"/>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -43559,7 +44501,11 @@
           <t>Medium: Design; project 'Can Typography Introduce Meaningful Friction to Resist Machine Readability &amp;amp; AI-Aided Surveillance?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J219" t="inlineStr"/>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -43599,7 +44545,11 @@
           <t>Medium: Painting/Drawing; project 'To Live Out The Name And to Perform Some Had'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J220" t="inlineStr"/>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -43639,7 +44589,11 @@
           <t>Medium: Painting/Drawing; project 'The Memetics of Generative AI Tools'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -43679,7 +44633,11 @@
           <t>Medium: Fiber and Material Arts; project 'Ritual'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J222" t="inlineStr"/>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -43719,7 +44677,11 @@
           <t>Medium: Sculpture; project 'Watermarks'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J223" t="inlineStr"/>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -43759,7 +44721,11 @@
           <t>Medium: Sculpture; project 'What Remains in the Hand'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J224" t="inlineStr"/>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -43799,7 +44765,11 @@
           <t>Medium: Design; project 'Lossy Greetings'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -43839,7 +44809,11 @@
           <t>Medium: Design; project 'CHANG HO: Structure as Identity'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J226" t="inlineStr"/>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -43879,7 +44853,11 @@
           <t>Medium: Design; project 'What's That Smell?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr"/>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -43919,7 +44897,11 @@
           <t>Medium: Fiber and Material Arts; project 'Supercalifragilisticexpialidocious'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J228" t="inlineStr"/>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -43959,7 +44941,11 @@
           <t>Medium: Sculpture; project 'Holding Time'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J229" t="inlineStr"/>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -43999,7 +44985,11 @@
           <t>Medium: Sculpture; project 'Lulu Lamp'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J230" t="inlineStr"/>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -44039,7 +45029,11 @@
           <t>Medium: Design; project 'We Love Repetitive Beats'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr"/>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -44079,7 +45073,11 @@
           <t>Medium: Design; project 'EyeSeeYou'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J232" t="inlineStr"/>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -44119,7 +45117,11 @@
           <t>Medium: Design; project 'A Line Out The Window: On Dreaming and Remembering'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J233" t="inlineStr"/>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -44159,7 +45161,11 @@
           <t>Medium: Design; project 'P.A.R.X - Physically Absorbing Reality eXtension'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J234" t="inlineStr"/>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -44199,7 +45205,11 @@
           <t>Medium: Sculpture; project 'Metamorphosis'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J235" t="inlineStr"/>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -44239,7 +45249,11 @@
           <t>Medium: Design; project 'Temple of the Lady Sun'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J236" t="inlineStr"/>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -44279,7 +45293,11 @@
           <t>Medium: Sculpture; project 'It’s In There Somewhere'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J237" t="inlineStr"/>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -44319,7 +45337,11 @@
           <t>Medium: Painting/Drawing; project 'The Idiot is Transcendent.'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J238" t="inlineStr"/>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -44359,7 +45381,11 @@
           <t>Medium: Fiber and Material Arts; project 'My Imagined Wedding'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J239" t="inlineStr"/>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -44399,7 +45425,11 @@
           <t>Medium: Fiber and Material Arts; project '"The Show Must Go On"'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J240" t="inlineStr"/>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -44439,7 +45469,11 @@
           <t>Medium: Fiber and Material Arts; project 'The Shape of A Spell'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J241" t="inlineStr"/>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -44479,7 +45513,11 @@
           <t>Medium: Fiber and Material Arts; project 'Portable Homelands'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J242" t="inlineStr"/>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -44519,7 +45557,11 @@
           <t>Medium: 2D/3D Animation; project 'Doll Searching'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J243" t="inlineStr"/>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -44559,7 +45601,11 @@
           <t>Medium: Design; project 'How Do You See The Poem?'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J244" t="inlineStr"/>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -44599,7 +45645,11 @@
           <t>Medium: Fiber and Material Arts; project 'Muddy Puddles'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J245" t="inlineStr"/>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -44639,7 +45689,11 @@
           <t>Medium: Painting/Drawing; project 'The Anatomy of a Gathering'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr"/>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -44679,7 +45733,11 @@
           <t>Medium: Filmmaking; project 'Do Not Upload'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J247" t="inlineStr"/>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -44719,7 +45777,11 @@
           <t>Medium: Design; project 'Inheritance in Knucklebones: An Autoethnography of Intergenerational Trauma'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J248" t="inlineStr"/>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -44759,7 +45821,11 @@
           <t>Medium: Design; project 'To Notice or Not to Notice'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J249" t="inlineStr"/>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -44799,7 +45865,11 @@
           <t>Medium: Fiber and Material Arts; project '“Then which of your Lord’s favours will you both deny?”'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J250" t="inlineStr"/>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -44839,7 +45909,11 @@
           <t>Medium: Painting/Drawing; project 'CSM MA Fine Art: Digital 2024-2026'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J251" t="inlineStr"/>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -44879,7 +45953,11 @@
           <t>Medium: Painting/Drawing; project '~Digital Genesis: 1999!**'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -44919,7 +45997,11 @@
           <t>Medium: Painting/Drawing; project 'Ink Narratives: Landscape, Memory and Place'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J253" t="inlineStr"/>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -44959,7 +46041,11 @@
           <t>Medium: Design; project 'Peter Mancuso Was Shot at 3:15 / The Afterlife of a Photograph'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J254" t="inlineStr"/>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -44999,7 +46085,11 @@
           <t>Medium: Design; project 'Genyuan #1 (Home Sweet Home)'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -45039,7 +46129,11 @@
           <t>Medium: Design; project 'Touch Grass'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -45079,7 +46173,11 @@
           <t>Medium: Fiber and Material Arts; project 'Contrada'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J257" t="inlineStr"/>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -45119,7 +46217,11 @@
           <t>Medium: Design; project 'Publishing Through Camouflage'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J258" t="inlineStr"/>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -45159,7 +46261,11 @@
           <t>Medium: Sculpture; project 'What We Leave Behind'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J259" t="inlineStr"/>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -45199,7 +46305,11 @@
           <t>Medium: Sculpture; project 'Now twilight lets her curtain down and pins it with a star'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -45239,7 +46349,11 @@
           <t>Medium: Fiber and Material Arts; project 'A sense of home'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J261" t="inlineStr"/>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -45279,7 +46393,11 @@
           <t>Medium: Fiber and Material Arts; project 'Chromatic Dialogues'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J262" t="inlineStr"/>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -45319,7 +46437,11 @@
           <t>Medium: Design; project 'Mist and Myths - An Illustrated Book About Slovenian Folklore'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -45359,7 +46481,11 @@
           <t>Medium: Design; project 'Inherited Memories'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J264" t="inlineStr"/>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -45399,7 +46525,11 @@
           <t>Medium: Design; project 'This Too shall Pass : A Tasting Menu'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J265" t="inlineStr"/>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -45439,7 +46569,11 @@
           <t>Medium: Sculpture; project 'Before It Fades'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J266" t="inlineStr"/>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -45479,7 +46613,11 @@
           <t>Medium: Sculpture; project 'Making Patterns'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -45519,7 +46657,11 @@
           <t>Medium: Design; project 'Keep Calm and Mend Project'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J268" t="inlineStr"/>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -45559,7 +46701,11 @@
           <t>Medium: Design; project 'Ocean Pollution Marine Animals vs Plastic'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J269" t="inlineStr"/>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -45599,7 +46745,11 @@
           <t>Medium: Fiber and Material Arts; project 'Identification and Desire'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -45639,7 +46789,11 @@
           <t>Medium: Sculpture; project 'From Which All Things Grow'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J271" t="inlineStr"/>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -45679,7 +46833,11 @@
           <t>Medium: Design; project 'Sending Love to Home and Home to Love'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -45719,7 +46877,11 @@
           <t>Medium: Fashion; project 'Mono No Aware'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr"/>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -45759,7 +46921,11 @@
           <t>Medium: Fiber and Material Arts; project 'The Old Man and The Sea'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr"/>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -45799,7 +46965,11 @@
           <t>Medium: Painting/Drawing; project 'Living Afterwards'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr"/>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -45839,7 +47009,11 @@
           <t>Medium: Sculpture; project 'Isabella Shinder'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J276" t="inlineStr"/>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -45879,7 +47053,11 @@
           <t>Medium: Sculpture; project 'Homegrown Sentiment'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J277" t="inlineStr"/>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -45919,7 +47097,11 @@
           <t>Medium: Fiber and Material Arts; project 'Indigo Lace, Patching Flowers'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -45959,7 +47141,11 @@
           <t>Medium: Design; project 'Perhaps I'm Meant to Hide This Way'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J279" t="inlineStr"/>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -45999,7 +47185,11 @@
           <t>Medium: Design; project 'The Invisible Threads of Computation'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J280" t="inlineStr"/>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -46039,7 +47229,11 @@
           <t>Medium: Design; project 'Print Politics Music, From 1976 to 1988'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr"/>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -46079,7 +47273,11 @@
           <t>Medium: Fiber and Material Arts; project 'Chroma-Fair'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr"/>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -46119,7 +47317,11 @@
           <t>Medium: Fashion; project 'Elle se souvient de tout, les parfums les couleurs'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J283" t="inlineStr"/>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -46159,7 +47361,11 @@
           <t>Medium: Design; project 'Lost and Found: Reclaiming Cultural Identity for Chinese Diasporic Women'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr"/>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -46199,7 +47405,11 @@
           <t>Medium: Painting/Drawing; project 'Even So, I Fed the Bird'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J285" t="inlineStr"/>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -46239,7 +47449,11 @@
           <t>Medium: Design; project 'River Fleet Interpretive Trail'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr"/>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -46279,7 +47493,11 @@
           <t>Medium: Fashion; project 'Polly Parker'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J287" t="inlineStr"/>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -46319,7 +47537,11 @@
           <t>Medium: Design; project 'Our Islands of Rhythms'; email found via mailto: link on UAL Showcase profile page</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:J288"/>
@@ -46328,6 +47550,222 @@
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="H6:H288" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Alfred University press releases and event pages naming 2026 and 2025 MFA Thesis Shows (Ceramic Art, Painting, Sculpture-Dimensional Studies, Electronic Integrated Arts). The original per-student thesis subpage system this project's source research relied on (thesis-exhibits/{year}/mfa/{lastname}/) has since been retired — every such URL now redirects to a generic photo-gallery hub with no consolidated roster, so this is a known-partial cohort pieced together from press releases and search-indexed event pages, not a single clean source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.alfred.edu/about/news/pressreleases/general/2026/nyscc-at-alfred-university-set-to-host-2026-mfa-thesis-shows.cfm (and 1 more 2026 press release, plus the 2025 MFA Thesis Exhibitions event calendar page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>sent_to_nitya</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:J6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Cornell AAP (College of Architecture, Art, and Planning) event pages for several small named MFA/BFA thesis group shows — Cornell's Department of Art does not publish one consolidated roster; cohorts are split across many 5-10 person exhibitions (MFA Image Text 'SELF/ASSEMBLY', MFA Creative Visual Arts, BFA 'Thesis Group Exhibition', 'Space of Becoming', 'Senior B.F.A. Thesis Exhibition', 'with a trace'). 2 more 2026 BFA sub-shows (FLEXION, 'North, South, East, West') referenced in search results but their pages were never located, so those names are a known gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://aap.cornell.edu/events/beyond-aap/m-f-a-image-text-26-thesis-show-self-assembly/ (and 5 more aap.cornell.edu event pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>sent_to_nitya</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:J6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -46374,6 +47812,330 @@
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Accessed: 2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>sent_to_nitya</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:J6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: UT Austin Visual Arts Center (utvac.org) event pages for the Studio Art MFA Thesis Exhibitions (2025 'Acceleration Without Arrival', 2026 'Half a Second or Less') and the 2026 Senior Art Exhibition ('Proof of Life') — each a single clean, complete roster page, the highest-yield source among the 5 schools added in this pass. A separate 2026 Design MFA show ('Known Otherwise', School of Design and Creative Technologies) was deliberately excluded as a different department outside this project's medium scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://utvac.org/event/proof-life-2026-senior-art-exhibition (and 2 more utvac.org event pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>sent_to_nitya</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:J6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: Cooper Union 'Class of 2026: In Their Own Words' feature article — the only 2 students explicitly confirmed as School of Art via an 'A'26' suffix. Cooper Union's annual End of Year Show has no roster page at all (names attributed by tradition only) and its opening-night photo gallery mixes all 3 schools (Architecture/Art/Engineering) together with no reliable way to isolate Art students without an explicit suffix — ~20 other names seen in photo captions were excluded as either confirmed non-Art or unverifiable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://cooper.edu/about/news/class-2026-their-own-words</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>graduation_year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>portfolio_url</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>college</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>contacted</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>sent_to_nitya</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:J6"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source: SCAD Thesis Digital Collection (library.scad.edu), a static/plain-HTML library catalog covering 50+ programs since Fall 2010 (MFA) / Spring 2020 (undergrad) — scoped to 2025-2026 only, matching this project's convention for every other school (current/recent cohorts, not full historical archives). 11 of SCAD's 50+ programs map to this project's in-scope mediums: Painting, Illustration, Printmaking (-&gt; Painting/Drawing), Sculpture, Fibers (-&gt; Fiber and Material Arts), Photography, Animation (-&gt; 2D/3D Animation), Film &amp; Television (-&gt; Filmmaking), Graphic Design (-&gt; Design), User Experience (UX) Design (-&gt; UI/UX Design), Fashion. Scraped via a purpose-built script (scad_scraper.py) since the catalog is far too large to browse manually (486 total Painting results alone, back to 2010).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://library.scad.edu/screens/theses.html (11 saved-search URLs, one per in-scope program)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-15</t>
         </is>
       </c>
     </row>
@@ -58847,7 +60609,11 @@
           <t>Email found via web search (broader phrasing 'Debra Dowden-Crockett artist email' surfaced it — first-pass VCU-specific search missed it). Institutional address at her current faculty appointment, Old Dominion University Art Department, post-graduation; corroborated by ODU Art Department directory listing</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -58891,7 +60657,11 @@
           <t>Email found via web search (broader phrasing 'August Neuscheler artist email' surfaced it). Correction: aneuscheler.info WAS the right site after all — a deeper page (neuscheler.shtml, not the bare homepage checked in the first pass) shows 'alexander august canossa neuscheler, richmond, va' with this email, verified in raw HTML</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -58935,7 +60705,11 @@
           <t>Email confirmed by user (portfolio site ayakhalife.com, JS-rendered Readymag site, personal email surfaced via 'Reach out' mailto link only visible on hover — not captured by automated fetch/crawl4ai)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -58979,7 +60753,11 @@
           <t>Email found via web search (own site rebeccaoh.com/about, verified in raw HTML: 'Feel free to e-mail the artist at rebeccaohart@gmail.com')</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -59023,7 +60801,11 @@
           <t>Email found via web search (VCU School of the Arts directory page, verified in raw HTML)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -59067,7 +60849,11 @@
           <t>Email found via web search (own site tynaontko.com/contact, address was obfuscated as 'ontkotyna(at)gmail(dot)com' in page text, deobfuscated)</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -59111,7 +60897,11 @@
           <t>Email confirmed by user (own site brooklin-studio.com — site's TLS certificate is expired server-side, blocking automated fetch, but user independently confirmed the address is correct; site content confirms ceramics/textiles, Richmond VA + Louisville KY)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -59155,7 +60945,11 @@
           <t>Email found via web search (own site mollygarrett.com/contact, address was obfuscated as 'hi [at] mollygarrett.com' in page text, deobfuscated)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -59195,7 +60989,11 @@
           <t>Email confirmed by user. CAUTION — name-collision flag: this exact address independently traces via search to a CV PDF for a different, well-documented Alex Bacon (art historian/curator, ex-Princeton Curatorial Associate, London/NY based), not to our Richmond VA painting MFA student (Alexander Kunin Bacon, b. 1995 Denver). Used per explicit user confirmation despite the mismatch in what's independently verifiable — worth a second look if this bounces</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -59239,7 +61037,11 @@
           <t>Email found via web search (own site duvalceramics.ca/contact, JS-rendered — found via interactive Playwright probe of the contact form page)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:J15"/>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx: 43 new emails from Cooper Union, Alfred, Cornell, UT Austin
Mirrors main@f9d32f2 -- Cooper Union 2/2 complete, Alfred 8/14, Cornell
11/39, UT Austin 14/78, found via Serper/Google search.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -68,10 +68,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'BGSU'!$A$5:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'CalArts Animation'!$A$5:$J$256</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'UAL Central Saint Martins'!$A$5:$J$288</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Alfred University'!$A$5:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Cornell'!$A$5:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'UT Austin'!$A$5:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Cooper Union'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Alfred University'!$A$5:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Cornell'!$A$5:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'UT Austin'!$A$5:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Cooper Union'!$A$5:$J$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'SCAD'!$A$5:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47563,7 +47563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -47651,13 +47651,365 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Amanda Gentry</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>studio@amandagentry.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Ceramic Art</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>http://www.amandagentry.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release (Fosdick-Nelson Gallery, opened April 4 2026). Email found via web search (own site amandagentry.com/about, verified in raw HTML mailto: link)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Max Heaton</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>maxheaton1@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.maxheaton.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release (Fosdick-Nelson Gallery, opened April 4 2026). Email found via web search (own site maxheaton.com bio section, verified in raw HTML mailto: link)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hazel Liu</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>yl25@alfred.edu</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Electronic Integrated Arts</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.alfred.edu/about/news/pressreleases/general/2026/nyscc-at-alfred-university-set-to-host-2026-mfa-thesis-shows.cfm</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release (Turner Gallery, opened April 4 2026). Email confirmed by user via Google AI Overview search. Alfred student-email initials ('yl') don't obviously match 'Hazel Liu' -- possibly a given/legal name difference (e.g. a Chinese given name starting with Y) -- used per user confirmation</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Yuxuan Wang</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fishywang@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Electronic Integrated Arts</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.alfred.edu/about/news/pressreleases/general/2026/nyscc-at-alfred-university-set-to-host-2026-mfa-thesis-shows.cfm</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release (Turner Gallery, opened April 4 2026). Email confirmed by user via Google AI Overview search. CAUTION -- name-collision flag: this exact address independently traces via this tool's search to a different, well-documented Yuxuan Wang (software developer/technologist, b. 1983 Wuhan, own site wang.yuxuan.org), not obviously our Alfred MFA art student. Used per explicit user confirmation despite the mismatch -- worth a second look if this bounces</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ignacio Luera</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Luera36@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Painting</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://ignacioluera.my.canva.site</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release (joint exhibition 'Homebody' with Justin Donica, opened April 11 2026). Email found via web search, verified in raw HTML on own site (ignacioluera.my.canva.site); Instagram @zer0logic bio confirms 'Painter / BFA at TSU / MA at TC Columbia U / MFA at Alfred U. '26'</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GH Wood</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ogwood03@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Ceramic Art</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://oghwood.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release (opened April 11 2026). Email found via web search (own site oghwood.com/new-page, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Marita Manson</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>maritamanson@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA Ceramic Art</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://maritamanson.com/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Name from 2026 MFA Thesis Shows press release ('The Call is Coming from Inside the House', Fosdick-Nelson Gallery, May 8-16 2026). Email found via Serper/Google search (her own Instagram @marita.manson bio text: 'send me a screen shot... to my email- maritamanson@gmail.com')</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Toomas Toomepuu</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>toomepuut@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA Sculpture-Dimensional Studies</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.sayhito-atlas.com/article/toomas-toompepuu</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Alfred University</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Name from 2025 MFA Thesis Exhibitions event page. Email found via Serper/Google search, listed directly on a sayhito-atlas.com feature article about his work. Own site (toomastoomepuu.com/about) still DNS-unreachable by this tool's fetchers, not checked directly</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J6"/>
+  <autoFilter ref="A5:J13"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -47671,7 +48023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -47759,13 +48111,497 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Smith Galtney</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>smithg@bakeryphoto.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Image Text</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>http://smithgaltney.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name from MFA Image Text '26 thesis show 'SELF/ASSEMBLY'. Email found via Serper/Google search on his Bakery Photo Collective core-member bio page, verified in raw HTML. Maine-based photographer/writer/storyteller</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jacquelyn Johnson</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>jacjohnsoninfo@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Image Text</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://jacjohnson.info/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name from MFA Image Text '26 thesis show 'SELF/ASSEMBLY'. Email found via Serper/Google search (own site jacjohnson.info/Info-Contact, verified in raw HTML, explicitly labeled 'MFA Candidate in Image Text at Cornell University')</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jared Radin</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jared@r4d1n.net</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Image Text</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://r4d1n.net/about</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Name from MFA Image Text '26 thesis show 'SELF/ASSEMBLY'. Email found via Serper/Google search (own site r4d1n.net/about, verified in raw HTML, explicitly labeled 'current MFA candidate in Image Text at Cornell University')</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Joseph Rafferty III</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>jar652@cornell.edu</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Image Text</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://josephrafferty.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Name from MFA Image Text '26 thesis show 'SELF/ASSEMBLY'. Email found via Serper/Google search (own site josephrafferty.com, verified in raw HTML, real Cornell institutional address)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carla Rangel García</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>rangel.g.carla@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Creative Visual Arts</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://carlarangelgarcia.com/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Name from MFA Creative Visual Arts '26 cohort (search-indexed). Email found via Serper/Google search (own site carlarangelgarcia.com/information, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Onome Olotu</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>studio.onomeolotu@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Creative Visual Arts</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://onomeolotu.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Name from MFA Creative Visual Arts '26 cohort. Email found via Serper/Google search, quoted directly in her Instagram bio (@onome_daniella_olotu: 'Artist Email: studio.onomeolotu@gmail.com DM for enquiries') -- not independently re-verified via raw HTML fetch since Instagram bios aren't fetchable by this tool, but the search snippet quotes it as an explicit self-labeled contact email</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sandy Wang</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sandywang1120@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA Creative Visual Arts</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://sandywang00.com/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Name from MFA Creative Visual Arts '26 cohort (full name Yun Hsiang (Sandy) Wang, Taiwanese interdisciplinary artist). Email found via Serper/Google search (own site sandywang00.com/info, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sheila Novak</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SheilaNovakStudios@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA Creative Visual Arts</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://sheilanovak.com/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Name from MFA Creative Visual Arts '26 cohort. Email found via Serper/Google search (own site sheilanovak.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sally Yu</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>jy652@cornell.edu</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/events/exhibition/thesis-group-exhibition/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Name from BFA '25 Senior Thesis 'Thesis Group Exhibition' (9 seniors). Email (full name Daeum Sally Yu) found via Serper/Google search, repeated across multiple Cornell AAP Instagram posts as her contact ('Feel free to email jy652@cornell.edu')</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lena Park</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>lp346@cornell.edu</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.lena-park.com/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Name from BFA '25 Senior Thesis 'Thesis Group Exhibition'; also appears in 'Space of Becoming' sub-show. Email found via Serper/Google search (own site lena-park.com/about and her LinkedIn, both list lp346@cornell.edu)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Asuka Kurebayashi</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ak2245@cornell.edu</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BFA Fine Arts</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.asukakurebayashi.com/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Cornell</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Name from BFA '26 thesis sub-show 'with a trace'. Email found via Serper/Google search (own site asukakurebayashi.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J6"/>
+  <autoFilter ref="A5:J16"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -47887,7 +48723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -47975,13 +48811,629 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nathan Anthony</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nathan.anthony@utexas.edu</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.nathan-anthony.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name from 'Acceleration Without Arrival' 2025 Studio Art MFA Thesis Exhibition (14 grads, Visual Arts Center, April 18-May 10 2025). Email found via Serper/Google search on UT Austin's official Art and Art History faculty/directory page, verified in raw HTML (institutional address; also has a personal nathan.anthony.dd@gmail.com listed on his own site)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ben Copolillo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>copolillob@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.bencopolillo.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name from 'Acceleration Without Arrival' 2025 Studio Art MFA Thesis Exhibition. Email found via Serper/Google search (own site bencopolillo.com/info-copy, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Noah Dasho</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>noah.dasho@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.noahdasho.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Name from 'Acceleration Without Arrival' 2025 Studio Art MFA Thesis Exhibition. Email found via Serper/Google search (own site noahdasho.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Christian Hastad</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>christianhastad@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://christianhastad.com/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Name from 'Acceleration Without Arrival' 2025 Studio Art MFA Thesis Exhibition. Email found via Serper/Google search (own site christianhastad.com/profile, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tova Katzman</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>tovakatzman.studio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (Photography and Video)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.tovakatzman.com/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Name from 'Acceleration Without Arrival' 2025 Studio Art MFA Thesis Exhibition; discipline (photography/video) confirmed via a second-year MFA mention in search results. Email found via Serper/Google search (own site tovakatzman.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Selina Wagner</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>swagnerstudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MFA Studio Art (Painting and Drawing)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://selinawagner.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Name from 'Acceleration Without Arrival' 2025 Studio Art MFA Thesis Exhibition. Email found via Serper/Google search (own site selinawagner.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rosalyn Jewel Farney</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>rosalynfarney@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.rosalynfarney.com/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Name from 'Half a Second or Less' 2026 Studio Art MFA Thesis Exhibition (7 grads, photography/painting/print/sculpture, Visual Arts Center, April 17-May 9 2026). Email found via Serper/Google search (own site rosalynfarney.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Jo Kim</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>joannekim103@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://joanne-kim.com/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Name from 'Half a Second or Less' 2026 Studio Art MFA Thesis Exhibition. Email found via Serper/Google search (own site joanne-kim.com, verified in raw HTML; legal name likely Joanne Kim, BA from Central Saint Martins UAL)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nolan Zunk</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>nolan@nolanzunk.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://www.nolanzunk.com/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Name from 'Half a Second or Less' 2026 Studio Art MFA Thesis Exhibition. Email found via Serper/Google search, listed as 'Contact info' on his Facebook page (facebook.com/nolan.img) -- not independently re-verified in his own site's raw HTML (no visible mailto link there), but a reasonably solid source</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Josiah Brown</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>josiah.brown.oh@gmail.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.josiahbrownart.com/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Name from 'Proof of Life' 2026 Senior Art Exhibition. Email found via Serper/Google search (own site josiahbrownart.com/about-me, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jeongin Choi</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>jpaintingc@gmail.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.jeonginchoi.com/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Name from 'Proof of Life' 2026 Senior Art Exhibition. Email found via Serper/Google search (own site jeonginchoi.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gabrielle Dick</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Gabrielle.gbd@gmail.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.gabrielledick.com/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Name from 'Proof of Life' 2026 Senior Art Exhibition. Email found via Serper/Google search (own site gabrielledick.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Reese Ertel</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>reeseertel.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.reeseertelart.com/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Name from 'Proof of Life' 2026 Senior Art Exhibition. Email found via Serper/Google search (her TikTok bio @reeseertel.art, corroborated by her own site reeseertelart.com; not independently re-verified in the site's raw HTML)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Claire Fleming</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>claireflem02@gmail.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BFA Studio Art</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.claireflemingart.com/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>UT Austin</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Name from 'Proof of Life' 2026 Senior Art Exhibition. Email found via Serper/Google search (own site claireflemingart.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J6"/>
+  <autoFilter ref="A5:J19"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -47995,7 +49447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -48083,13 +49535,101 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Skye Jones</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>skyealgojones@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BFA Art (HSS minor: History and Theory of Art)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>http://skyejones.info/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cooper Union</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Name from 'Class of 2026: In Their Own Words' article; confirmed School of Art via 'A'26' suffix. Creates installations; exhibited work titled 'Ornamental Child'. Email found via Serper/Google search (own site skyejones.info/contact, verified in raw HTML), bio confirms film/photo work matching the 'Ornamental Child' Foundation Building show listing. Cooper Union's School of Art has no consolidated roster page (per tradition, work is attributed by artist name only, spread across annual End of Year Show photo captions mixing all 3 schools — Art/Architecture/Engineering — with no reliable way to distinguish School of Art students from the others without an explicit suffix)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Regina Cervantes Ellis</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>regina.ce@icloud.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BFA Art (HSS minor: History and Theory of Art)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.reginacervantes.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Cooper Union</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Name from 'Class of 2026: In Their Own Words' article; confirmed School of Art via 'A'26' suffix. Researched Mexican Restaurant Graphic Design via the Rhoda Lubalin Fellowship; exhibited work titled 'Sandia, Sanoche'. Email found via web search (own site reginacervantes.com, verified in raw HTML mailto: link)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J6"/>
+  <autoFilter ref="A5:J7"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Email discovery pass for SCAD: 67/367 confirmed (Film & TV, Animation, Illustration complete)
Individual per-name search + raw-HTML/self-declaration verification across
all 11 in-scope SCAD programs. Session added 27 new confirmed emails on top
of the earlier Fibers/Sculpture/Fashion/Photography/Graphic Design/Painting
pass, completing Film & Television (14/66), Animation (11/76), and
Illustration (11/93).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -72,7 +72,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Cornell'!$A$5:$J$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'UT Austin'!$A$5:$J$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Cooper Union'!$A$5:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'SCAD'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'SCAD'!$A$5:$J$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49643,7 +49643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -49731,13 +49731,2961 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Jannelly Herrera</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>jannellyherrera1126@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.jannellyherrera.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Pajara, An Investigation of the Feminine Experience'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site jannellyherrera.com/artist-biography, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sandra Iafrate</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>iafrate.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.sandraiafrate.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Portrait of Past and Present'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site sandraiafrate.com/about-artist, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rachel Korzeb</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rachelkorzeb@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.rachelkorzeb.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Imagination and Reality'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site rachelkorzeb.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Elise Le Gallo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>eliselegallo@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.leboulot.org/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Light is Like Water'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, corroborated across own site (leboulot.org, verified in raw HTML) and her own CV PDF</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sharon Potter</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>spotterartstudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/sharonpotterart/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'When 'Resilient' Becomes a Four-Letter Word: Living with the Aftermath'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed as Contact Info on her Facebook page, corroborated by a second Facebook page tagging 'Savannah College Of Art And Design'</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nikki Rakov</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>info@nikkirakovart.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.nikkirakovart.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'To Know, To Dare, To Keep Silent'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site nikkirakovart.com/artist-resume, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cristina Marietta Komaroff</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>c.komaroff@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.madamecristina.art/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Cristina's Gaze'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site madamecristina.art, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Shannon Meadows</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>shannonmeadowsfineart@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.shannonmeadows.com/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'On Our Own Terms'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own bio site shannonmeadows.com/about, verified in raw HTML; also self-published on her Instagram @shannonmeadows678 with a slightly different address, this one preferred as more authoritative)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Keshav Prasad</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>suryapsd000@gmail.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://artbykeshav.carrd.co/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Revelations of Food and History'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, quoted directly in the search snippet from his own site (artbykeshav.carrd.co, 'Enquiries via Email or Instagram. Email: suryapsd000@gmail...') -- not independently re-verified via raw HTML fetch since carrd.co content may be JS-rendered</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Evelyn Shoults</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>evelyn@bshoults.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.evelynshoults.com/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Daily Dose: Ritual, Recovery, and the Unheard Patient'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site evelynshoults.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Joanna Silver</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>joannapsilver@gmail.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.joannapaigesilver.com/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'What American Dream?'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site joannapaigesilver.com/about-me-4, verified in raw HTML; full name Joanna Paige Silver)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Denis Byrd</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>studio@denisbyrd.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.denisbyrd.com/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Sehnsucht: Longing and Joy in the Southern Landscape'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, quoted directly in the search snippet from his own site's shop page ('please email me for availability. studio@denisbyrd.com') -- his site is currently returning 404 on direct fetch (may be temporarily down), not independently re-verified via raw HTML</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hannah Grace Maki</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>studio@hannahgrace.art</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.hannahgrace.art/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'The Duality of Reality'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site hannahgrace.art/aboutme, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jazmin Marie Saunders</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>jazmarie.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://jazmarie.art/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Sucrose'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site jazmarie.art, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Connor Stelle</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>connorstelle@gmail.com</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Kingdom of Shadows: Reimagining Silent Horror Films Through Traditional Inking Techniques'; email verified in raw HTML on his own portfolio site connorstelleillustration.com</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Chani Alia Becker</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>chani@chanibecker.com</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Beneath the Surface: Depicting the Depths of Fairy Tales through Jungian-Psychology Informed Illustr'; email verified in raw HTML on her own portfolio site chanibecker.com contact page</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Juntang Xu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>juntangxustudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'The Use of White Space in Picture Books  A Study of Aesthetics and Narrative'; email self-declared in his own Instagram bio</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Jake Steven Czubinski</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>jakeczubinski@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Weyward Cove: Intersection of Cultural Identity and Queer Representation for Youth in Children's Tel'; email verified in raw HTML on his own portfolio site czubinski.myportfolio.com</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jordyn Goodman</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>jordyngoodman14@gmail.com</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Cyber Girls: Bringing to Life STEAM Interests in Children Through Toy Design'; email verified in raw HTML on her own portfolio site jordyngoodman.myportfolio.com</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wynter Malone</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>wynterartist@gmail.com</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Magnificent Moths: Representing the Beauty and Purpose of All in Nature'; email verified in raw HTML on her own portfolio site wynterartist.com contact page</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hollie Puterbaugh</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>hollieillu@gmail.com</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Layers of Meaning: Conceptual Devices in Contemporary Editorial Illustration'; email self-declared and corroborated across her own site hollieillu.com, Instagram bio, LinkedIn, and interview feature</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Maggie Stinauer</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>StinaCaliArt@gmail.com</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Story Telling: The Role of Conceptual Illustration in Society, and the Editorial Outlet'; email verified in raw HTML on her own portfolio site stinacali.com contact page (professional name "Stina Cali")</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Lai Wei</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>laiwei511@gmail.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Symbols in Illustration &amp; How They Affect Storytelling'; email verified in raw HTML on her own portfolio site laiwei21.com about page</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jiayi Zhang</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>jiayi6120@gmail.com</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'The Influence of Line Drawing in the Song Dynasty to Present Illustration Creation'; email verified in raw HTML on his own portfolio site jiayizhangtom.org contact page</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Richard Zhao</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>zgradecomics@gmail.com</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Cognition: Exploration of Character Archetypes and Symbolism Through the Lens of Environmental Desig'; email listed in structured "e:" contact field on official Applied Arts Magazine 2025 Student Awards winner page, directly attached to his name and SCAD</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Emma Adler</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>emmaadler1@gmail.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sculpture (SCAD)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.emmaadler.com/</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Medium: Sculpture; thesis title 'AMI: The Digital Representation of Women in Western Pop Culture'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site emmaadler.com/about-4, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Lusiana Morales Febo</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>lusiana.arte@gmail.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fibers (SCAD)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.lusianamorales.com</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Medium: Fiber and Material Arts; thesis title 'Earthtanglements: Reconnecting and Renewing Relationships with Our Environment'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (Voyage Savannah feature article, explicit Contact Info line, verified in raw page content)</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Melanee "Mel" Brown</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>itsmelbeephotography@gmail.com</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.melaneebrownmedia.com/</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Burney Road'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, self-declared in her own Instagram bio (introducing herself as 'Melanee Brown, a photographer and MFA candidate at SCAD Atlanta') and independently repeated when a separate account photo-credited her with the same handle -- her own site melaneebrownmedia.com only has a contact form, no direct mailto</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Kourtney Iman King</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>info@kourtneyiman.com</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/_kourtneyiman/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Soulaan Femme'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, matches her own domain name and repeated consistently across her Instagram bio and post captions as her direct inquiry contact</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Taylor Edgerton</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>edgertonphoto@gmail.com</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://tayloreedgerton.format.com/</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Book Under the Pew'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed in Instagram bio (@tayloreedgerton, 'available for work: edgertonphoto@gmail.com')</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hailey R. Kasper</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Hailey9Kasper@gmail.com</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://haileykasper.com/</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Anything Magazine'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site haileykasper.com/events, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Xavier Thompson</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>x.ix@gmail.com</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://xaviertylerthompson.com/</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'A Place Beyond the Pine'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site xaviertylerthompson.com/about-me-1, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DeAngelo Williams</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>navyskyphoto@gmail.com</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/navy_sky_photography/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Connections'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, explicit 'Contact Info' line in a Voyage ATL feature article ('Meet DeAngelo Williams of Navy Sky Photography'), matches his Instagram bio noting 'SCAD MFA Photography 2025'. NOTE: a WebFetch pass on the same article guessed a different, unverifiable deobfuscated address from a Cloudflare-protected mailto link -- not used, since it wasn't literal page text</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Zhiquan Zhao</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>zhzhao1230@gmail.com</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/zhiquanzhao_/</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Journey to the American Dream'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed in Instagram bio (@zhiquanzhao_, 'DM or Email for Bookings zhzhao1230@gmail.com', tagged #scad #scadphotography), matches his thesis exhibition blog post at the same name</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Lan Luo</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>lanluo@lanluoart.com</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Unknown Waiting : The Use of Visual Metaphor in 3D Animated Film'; email verified in raw HTML on her own portfolio site lanluoart.com about page</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sarah Via</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>sarahcvia@gmail.com</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Ranger Dave Enjoys a Quiet Evening : A Study in the Real and Unreal in Animated Media'; email verified in raw HTML on her own portfolio site sarahcvia.com (about + resume pages)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Yoona Hwang</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>yoonahwang.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Silence : Visualizing Sound through Hybrid Animation for Disability Advocacy and Inclusion'; email verified in raw HTML on her own portfolio site yoonahwang.com (about + contact pages); also self-declared as silence.film.official@gmail.com on her thesis film's therookies.co page</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Gabby Gillespie</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>gabbygillespie24@gmail.com</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'How the Animal Animated Film Recontextualizes Our Perception of History'; email verified in raw HTML on her own portfolio site gabbygillespieart.com</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Freddy Bendekgey</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>freddybendekgey@gmail.com</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Queer-Coded Lighting : How Lighting and Cinematography Can Subvert the Expectations of the Male Gaze'; email verified in raw HTML on his own portfolio site freddybendekgey.com</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Daniela Rumbaut</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>danielarumbaut@utexas.edu</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Chopin et Liszt : Hand-Painted Watercolor Textures for 3D Animation'; email verified in raw HTML on her own portfolio site danielarumbaut.myportfolio.com contact page (UT Austin .edu address, not SCAD -- listed as her own current contact)</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Drew Clark</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>drew.anne.clark@gmail.com</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Cure Haven Introduction'; email verified in raw HTML on her own portfolio site sodapopsketches.com</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Anindita Maturi</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>aninditamaturi.98@gmail.com</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Mamidi : The Fusion of 2D and 3D Animation to Enhance Storytelling and Aesthetic Appeal'; email verified in raw HTML on her own portfolio site (Wix)</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Iman Gadalla</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>imanmgadalla@gmail.com</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Animation as Therapy : The Power of Character Design and Narrative Art in Art Therapy'; email self-declared in her own Instagram post ("EMAIL ME AT IMANMGADALLA@GMAIL.COM")</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Mark J. Boone</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>mboone20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Dog Eat Dogma : Expressing the Parallels of Man and Canine Stereotyping Through Anthropomorphism'; email self-declared on his own LinkedIn profile (handle mboone20 matches address)</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Ian Anastas</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>itanastas@gmail.com</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'ConTempt Warning : Cartoony Comedic Musical Performance in the Context of Contemporary Social Media'; email self-declared in his own Instagram bio ("Open for work: itanastas@gmail.com")</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Zilyu Ye</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>zilyye20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Medium as Mirror : Investigating the Alignment of Reflexive Intent and Film Ontology in Independent'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, repeated verbatim (same exact address) across two separate Savannah Actors Facebook group casting-call posts for her SCAD thesis film</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sean Malady</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>august.starling@gmail.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'The Advancements and New Techniques in Low-Light Digital Cinematography'; email self-declared as "Sean Malady Email:" in his own crew casting-call posts, corroborated across 2 separate Facebook posts</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Adrianna Amy-Delgado</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>aplowd20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://www.scadproductionoffice.com/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Coming of Rage'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, on her own SCAD Production Office profile page ('Please reach out to me at aplowd20@student.scad.edu')</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pranav Abraham Varikad</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>pranav810x@gmail.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://pranavabraham.com/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'What Girls Want'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site pranav810x.wixsite.com/pranavabraham, 'Get in touch today', quoted directly in search snippet)</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Koyna Mitra</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>kmitra20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://www.scadproductionoffice.com/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Identity Negotiation in Liminality : Migration, Gender, and Selfhood in Bollywood and Diasporic Cine'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, on her own SCAD Production Office profile page (structured Email field)</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Keishla Marie Oquendo</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>xkeishla@gmail.com</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DCACWuEJBcg/</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Chrysalis'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed in her Instagram bio; identity corroborated by a Voyage ATL feature article ('Meet Keishla Oquendo of Atlanta')</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Nguyen Brian</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>bnguye24@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://www.scadproductionoffice.com/</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'A Technical Overview of Selecting Lights while Dealing with Multiple Skin Tones'; from SCAD Thesis Digital Collection (library.scad.edu). Full name Brian Nguyen. Email found via Serper/Google search, on his own SCAD Production Office profile page (structured Email field)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fatima Diallo</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Fdiallo33@gmail.com</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/__fatimadiallo/</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Queer Film in Africa'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed on her own Instagram post ('Website: Vimeo.com/fatimadiallo Instagram: @_fatimadiallo Other: Fdiallo33@gmail.com')</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Noah Trainor</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>nbtrainor21@gmail.com</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://www.noahtrainor.com/</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Subverting Cinematic Depictions of Toxic Masculinity in the Films of Noah Baumbach'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site noahtrainor.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Becca Robinson</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>srobin34@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://filmwithbecca.com/</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'You Can't Joke About That : The Creation of Inheritance, a Short Film Inspired by a Study of the Psy'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, on her own SCAD Production Office profile page (structured Email field)</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Scott Joseph Moore</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>smartcastings@live.com</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Collective Consciousness and the Art of Film Making'; email self-declared in his own YouTube video description with his name and LinkedIn attached</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Cache Jill Capuyan</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>afterthecreditsroll.films@gmail.com</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'To Whom It May Concern : Illuminating Survivors of Male Domestic Violence and Exploring their Dismis'; email verified in raw HTML on her own portfolio site afterthecreditsroll.weebly.com contact page</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Esteban Larach</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>estebanlarachg@gmail.com</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Moral Dilemmas in Thrillers : The Consequences of Split-Second Decisions'; email verified in raw HTML on his own portfolio site estebanlarach.com contact page</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Yulin Chen</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>yulin@redpavilionfilms.com</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Love, Tears, and Choice'; email verified in raw HTML on her own studio site redpavilionfilms.com/about-1 (Producer bio)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Mingxuan Duan</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>duanmx1717@gmail.com</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://www.mingxuan.design/</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Designing for Motivation: Transforming Procrastination with Graphic Design Strategies'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site mingxuan.design/contact, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Trevor Kimathi Mugambi</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>trevormugambi@gmail.com</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.trevormugambi.com/</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Enhancing African Representation in the Graphic Design Industry'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site trevormugambi.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Caroline Schwarm</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>caroline.schwarm@gmail.com</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://www.carolineschwarm.com/</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Mirror, Mirror on the Screen'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site carolineschwarm.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Xiaoyue Shen</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>neosoulclub88@gmail.com</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://www.xiaoyueshen.com/</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Visualizing Secondary Memory Through Graphic Design'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, read directly from her own resume PDF (freight.cargo.site link, PDF text extracted and verified)</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Sia Tyagi</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>sia.s.tyagi@gmail.com</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://siatyagi.com/</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Between Worlds: Redefining Design for Hybrid Realities'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site siatyagi.com/contact, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Rupal Panwar</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>rupal26panwar@gmail.com</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Fashion (SCAD)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://www.rupalpanwar.com/</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Medium: Fashion; thesis title 'Creating Cultural Belonging Among Immigrants Through the Lens of Kashmir'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site rupalpanwar.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Jiani Hu</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>jiani4942@gmail.com</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Fashion (SCAD)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://www.jianihu.com/</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Medium: Fashion; thesis title 'In Between Black and White: The Fashion Potential of Yin-Yang Philosophy in the West'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site jianihu.com/resume, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Isaac Yu</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>isaac890302@gmail.com</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Fashion (SCAD)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://www.isaac-yu.art/</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Medium: Fashion; thesis title 'Who Kills My Freedom'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, corroborated on two sources (own site isaac-yu.art contact form, verified in raw HTML; also listed as 'Press Contact' on his Instagram @imisaacyu)</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J6"/>
+  <autoFilter ref="A5:J72"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update master_students_with_email.xlsx: SCAD email discovery pass (67/367)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
+++ b/Dezi Art Prize Student Data Scraping/master_students_with_email.xlsx
@@ -72,7 +72,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Cornell'!$A$5:$J$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'UT Austin'!$A$5:$J$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Cooper Union'!$A$5:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'SCAD'!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'SCAD'!$A$5:$J$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49643,7 +49643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -49731,13 +49731,2961 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Jannelly Herrera</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>jannellyherrera1126@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.jannellyherrera.com/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Pajara, An Investigation of the Feminine Experience'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site jannellyherrera.com/artist-biography, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sandra Iafrate</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>iafrate.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.sandraiafrate.com/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Portrait of Past and Present'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site sandraiafrate.com/about-artist, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rachel Korzeb</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rachelkorzeb@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.rachelkorzeb.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Imagination and Reality'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site rachelkorzeb.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Elise Le Gallo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>eliselegallo@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.leboulot.org/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Light is Like Water'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, corroborated across own site (leboulot.org, verified in raw HTML) and her own CV PDF</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sharon Potter</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>spotterartstudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/sharonpotterart/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'When 'Resilient' Becomes a Four-Letter Word: Living with the Aftermath'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed as Contact Info on her Facebook page, corroborated by a second Facebook page tagging 'Savannah College Of Art And Design'</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nikki Rakov</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>info@nikkirakovart.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.nikkirakovart.com/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'To Know, To Dare, To Keep Silent'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site nikkirakovart.com/artist-resume, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cristina Marietta Komaroff</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>c.komaroff@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.madamecristina.art/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Cristina's Gaze'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site madamecristina.art, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Shannon Meadows</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>shannonmeadowsfineart@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.shannonmeadows.com/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'On Our Own Terms'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own bio site shannonmeadows.com/about, verified in raw HTML; also self-published on her Instagram @shannonmeadows678 with a slightly different address, this one preferred as more authoritative)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Keshav Prasad</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>suryapsd000@gmail.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://artbykeshav.carrd.co/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Revelations of Food and History'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, quoted directly in the search snippet from his own site (artbykeshav.carrd.co, 'Enquiries via Email or Instagram. Email: suryapsd000@gmail...') -- not independently re-verified via raw HTML fetch since carrd.co content may be JS-rendered</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Evelyn Shoults</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>evelyn@bshoults.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.evelynshoults.com/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Daily Dose: Ritual, Recovery, and the Unheard Patient'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site evelynshoults.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Joanna Silver</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>joannapsilver@gmail.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.joannapaigesilver.com/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'What American Dream?'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site joannapaigesilver.com/about-me-4, verified in raw HTML; full name Joanna Paige Silver)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Denis Byrd</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>studio@denisbyrd.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.denisbyrd.com/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Sehnsucht: Longing and Joy in the Southern Landscape'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, quoted directly in the search snippet from his own site's shop page ('please email me for availability. studio@denisbyrd.com') -- his site is currently returning 404 on direct fetch (may be temporarily down), not independently re-verified via raw HTML</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hannah Grace Maki</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>studio@hannahgrace.art</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.hannahgrace.art/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'The Duality of Reality'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site hannahgrace.art/aboutme, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jazmin Marie Saunders</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>jazmarie.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Painting (SCAD)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://jazmarie.art/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Sucrose'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site jazmarie.art, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Connor Stelle</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>connorstelle@gmail.com</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Kingdom of Shadows: Reimagining Silent Horror Films Through Traditional Inking Techniques'; email verified in raw HTML on his own portfolio site connorstelleillustration.com</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Chani Alia Becker</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>chani@chanibecker.com</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Beneath the Surface: Depicting the Depths of Fairy Tales through Jungian-Psychology Informed Illustr'; email verified in raw HTML on her own portfolio site chanibecker.com contact page</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Juntang Xu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>juntangxustudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'The Use of White Space in Picture Books  A Study of Aesthetics and Narrative'; email self-declared in his own Instagram bio</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Jake Steven Czubinski</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>jakeczubinski@yahoo.com</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Weyward Cove: Intersection of Cultural Identity and Queer Representation for Youth in Children's Tel'; email verified in raw HTML on his own portfolio site czubinski.myportfolio.com</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jordyn Goodman</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>jordyngoodman14@gmail.com</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Cyber Girls: Bringing to Life STEAM Interests in Children Through Toy Design'; email verified in raw HTML on her own portfolio site jordyngoodman.myportfolio.com</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wynter Malone</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>wynterartist@gmail.com</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Magnificent Moths: Representing the Beauty and Purpose of All in Nature'; email verified in raw HTML on her own portfolio site wynterartist.com contact page</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hollie Puterbaugh</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>hollieillu@gmail.com</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Layers of Meaning: Conceptual Devices in Contemporary Editorial Illustration'; email self-declared and corroborated across her own site hollieillu.com, Instagram bio, LinkedIn, and interview feature</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Maggie Stinauer</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>StinaCaliArt@gmail.com</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Story Telling: The Role of Conceptual Illustration in Society, and the Editorial Outlet'; email verified in raw HTML on her own portfolio site stinacali.com contact page (professional name "Stina Cali")</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Lai Wei</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>laiwei511@gmail.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Symbols in Illustration &amp; How They Affect Storytelling'; email verified in raw HTML on her own portfolio site laiwei21.com about page</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jiayi Zhang</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>jiayi6120@gmail.com</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'The Influence of Line Drawing in the Song Dynasty to Present Illustration Creation'; email verified in raw HTML on his own portfolio site jiayizhangtom.org contact page</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Richard Zhao</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>zgradecomics@gmail.com</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Illustration (SCAD)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Medium: Painting/Drawing; thesis title 'Cognition: Exploration of Character Archetypes and Symbolism Through the Lens of Environmental Desig'; email listed in structured "e:" contact field on official Applied Arts Magazine 2025 Student Awards winner page, directly attached to his name and SCAD</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Emma Adler</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>emmaadler1@gmail.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sculpture (SCAD)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.emmaadler.com/</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Medium: Sculpture; thesis title 'AMI: The Digital Representation of Women in Western Pop Culture'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site emmaadler.com/about-4, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Lusiana Morales Febo</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>lusiana.arte@gmail.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fibers (SCAD)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.lusianamorales.com</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Medium: Fiber and Material Arts; thesis title 'Earthtanglements: Reconnecting and Renewing Relationships with Our Environment'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (Voyage Savannah feature article, explicit Contact Info line, verified in raw page content)</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Melanee "Mel" Brown</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>itsmelbeephotography@gmail.com</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.melaneebrownmedia.com/</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Burney Road'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, self-declared in her own Instagram bio (introducing herself as 'Melanee Brown, a photographer and MFA candidate at SCAD Atlanta') and independently repeated when a separate account photo-credited her with the same handle -- her own site melaneebrownmedia.com only has a contact form, no direct mailto</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Kourtney Iman King</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>info@kourtneyiman.com</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/_kourtneyiman/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Soulaan Femme'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, matches her own domain name and repeated consistently across her Instagram bio and post captions as her direct inquiry contact</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Taylor Edgerton</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>edgertonphoto@gmail.com</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://tayloreedgerton.format.com/</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Book Under the Pew'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed in Instagram bio (@tayloreedgerton, 'available for work: edgertonphoto@gmail.com')</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hailey R. Kasper</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Hailey9Kasper@gmail.com</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://haileykasper.com/</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Anything Magazine'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site haileykasper.com/events, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Xavier Thompson</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>x.ix@gmail.com</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://xaviertylerthompson.com/</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'A Place Beyond the Pine'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site xaviertylerthompson.com/about-me-1, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DeAngelo Williams</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>navyskyphoto@gmail.com</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/navy_sky_photography/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Connections'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, explicit 'Contact Info' line in a Voyage ATL feature article ('Meet DeAngelo Williams of Navy Sky Photography'), matches his Instagram bio noting 'SCAD MFA Photography 2025'. NOTE: a WebFetch pass on the same article guessed a different, unverifiable deobfuscated address from a Cloudflare-protected mailto link -- not used, since it wasn't literal page text</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Zhiquan Zhao</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>zhzhao1230@gmail.com</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Photography (SCAD)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/zhiquanzhao_/</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Medium: Photography; thesis title 'Journey to the American Dream'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed in Instagram bio (@zhiquanzhao_, 'DM or Email for Bookings zhzhao1230@gmail.com', tagged #scad #scadphotography), matches his thesis exhibition blog post at the same name</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Lan Luo</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>lanluo@lanluoart.com</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Unknown Waiting : The Use of Visual Metaphor in 3D Animated Film'; email verified in raw HTML on her own portfolio site lanluoart.com about page</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sarah Via</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>sarahcvia@gmail.com</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Ranger Dave Enjoys a Quiet Evening : A Study in the Real and Unreal in Animated Media'; email verified in raw HTML on her own portfolio site sarahcvia.com (about + resume pages)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Yoona Hwang</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>yoonahwang.art@gmail.com</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Silence : Visualizing Sound through Hybrid Animation for Disability Advocacy and Inclusion'; email verified in raw HTML on her own portfolio site yoonahwang.com (about + contact pages); also self-declared as silence.film.official@gmail.com on her thesis film's therookies.co page</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Gabby Gillespie</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>gabbygillespie24@gmail.com</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'How the Animal Animated Film Recontextualizes Our Perception of History'; email verified in raw HTML on her own portfolio site gabbygillespieart.com</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Freddy Bendekgey</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>freddybendekgey@gmail.com</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Queer-Coded Lighting : How Lighting and Cinematography Can Subvert the Expectations of the Male Gaze'; email verified in raw HTML on his own portfolio site freddybendekgey.com</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Daniela Rumbaut</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>danielarumbaut@utexas.edu</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Chopin et Liszt : Hand-Painted Watercolor Textures for 3D Animation'; email verified in raw HTML on her own portfolio site danielarumbaut.myportfolio.com contact page (UT Austin .edu address, not SCAD -- listed as her own current contact)</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Drew Clark</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>drew.anne.clark@gmail.com</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Cure Haven Introduction'; email verified in raw HTML on her own portfolio site sodapopsketches.com</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Anindita Maturi</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>aninditamaturi.98@gmail.com</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Mamidi : The Fusion of 2D and 3D Animation to Enhance Storytelling and Aesthetic Appeal'; email verified in raw HTML on her own portfolio site (Wix)</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Iman Gadalla</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>imanmgadalla@gmail.com</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Animation as Therapy : The Power of Character Design and Narrative Art in Art Therapy'; email self-declared in her own Instagram post ("EMAIL ME AT IMANMGADALLA@GMAIL.COM")</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Mark J. Boone</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>mboone20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'Dog Eat Dogma : Expressing the Parallels of Man and Canine Stereotyping Through Anthropomorphism'; email self-declared on his own LinkedIn profile (handle mboone20 matches address)</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Ian Anastas</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>itanastas@gmail.com</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Animation (SCAD)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Medium: 2D/3D Animation; thesis title 'ConTempt Warning : Cartoony Comedic Musical Performance in the Context of Contemporary Social Media'; email self-declared in his own Instagram bio ("Open for work: itanastas@gmail.com")</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Zilyu Ye</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>zilyye20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Medium as Mirror : Investigating the Alignment of Reflexive Intent and Film Ontology in Independent'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, repeated verbatim (same exact address) across two separate Savannah Actors Facebook group casting-call posts for her SCAD thesis film</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sean Malady</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>august.starling@gmail.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'The Advancements and New Techniques in Low-Light Digital Cinematography'; email self-declared as "Sean Malady Email:" in his own crew casting-call posts, corroborated across 2 separate Facebook posts</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Adrianna Amy-Delgado</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>aplowd20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://www.scadproductionoffice.com/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Coming of Rage'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, on her own SCAD Production Office profile page ('Please reach out to me at aplowd20@student.scad.edu')</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pranav Abraham Varikad</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>pranav810x@gmail.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://pranavabraham.com/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'What Girls Want'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site pranav810x.wixsite.com/pranavabraham, 'Get in touch today', quoted directly in search snippet)</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Koyna Mitra</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>kmitra20@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://www.scadproductionoffice.com/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Identity Negotiation in Liminality : Migration, Gender, and Selfhood in Bollywood and Diasporic Cine'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, on her own SCAD Production Office profile page (structured Email field)</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Keishla Marie Oquendo</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>xkeishla@gmail.com</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DCACWuEJBcg/</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Chrysalis'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed in her Instagram bio; identity corroborated by a Voyage ATL feature article ('Meet Keishla Oquendo of Atlanta')</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Nguyen Brian</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>bnguye24@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://www.scadproductionoffice.com/</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'A Technical Overview of Selecting Lights while Dealing with Multiple Skin Tones'; from SCAD Thesis Digital Collection (library.scad.edu). Full name Brian Nguyen. Email found via Serper/Google search, on his own SCAD Production Office profile page (structured Email field)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fatima Diallo</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Fdiallo33@gmail.com</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/__fatimadiallo/</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Queer Film in Africa'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, listed on her own Instagram post ('Website: Vimeo.com/fatimadiallo Instagram: @_fatimadiallo Other: Fdiallo33@gmail.com')</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Noah Trainor</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>nbtrainor21@gmail.com</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://www.noahtrainor.com/</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Subverting Cinematic Depictions of Toxic Masculinity in the Films of Noah Baumbach'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site noahtrainor.com/about, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Becca Robinson</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>srobin34@student.scad.edu</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://filmwithbecca.com/</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'You Can't Joke About That : The Creation of Inheritance, a Short Film Inspired by a Study of the Psy'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, on her own SCAD Production Office profile page (structured Email field)</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Scott Joseph Moore</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>smartcastings@live.com</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Collective Consciousness and the Art of Film Making'; email self-declared in his own YouTube video description with his name and LinkedIn attached</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Cache Jill Capuyan</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>afterthecreditsroll.films@gmail.com</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'To Whom It May Concern : Illuminating Survivors of Male Domestic Violence and Exploring their Dismis'; email verified in raw HTML on her own portfolio site afterthecreditsroll.weebly.com contact page</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Esteban Larach</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>estebanlarachg@gmail.com</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Moral Dilemmas in Thrillers : The Consequences of Split-Second Decisions'; email verified in raw HTML on his own portfolio site estebanlarach.com contact page</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Yulin Chen</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>yulin@redpavilionfilms.com</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Film &amp; Television (SCAD)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://library.scad.edu/screens/theses.html</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Medium: Filmmaking; thesis title 'Love, Tears, and Choice'; email verified in raw HTML on her own studio site redpavilionfilms.com/about-1 (Producer bio)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Mingxuan Duan</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>duanmx1717@gmail.com</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://www.mingxuan.design/</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Designing for Motivation: Transforming Procrastination with Graphic Design Strategies'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site mingxuan.design/contact, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Trevor Kimathi Mugambi</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>trevormugambi@gmail.com</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.trevormugambi.com/</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Enhancing African Representation in the Graphic Design Industry'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site trevormugambi.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Caroline Schwarm</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>caroline.schwarm@gmail.com</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://www.carolineschwarm.com/</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Mirror, Mirror on the Screen'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site carolineschwarm.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Xiaoyue Shen</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>neosoulclub88@gmail.com</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://www.xiaoyueshen.com/</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Visualizing Secondary Memory Through Graphic Design'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, read directly from her own resume PDF (freight.cargo.site link, PDF text extracted and verified)</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Sia Tyagi</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>sia.s.tyagi@gmail.com</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Graphic Design (SCAD)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://siatyagi.com/</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Medium: Design; thesis title 'Between Worlds: Redefining Design for Hybrid Realities'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site siatyagi.com/contact, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Rupal Panwar</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>rupal26panwar@gmail.com</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Fashion (SCAD)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://www.rupalpanwar.com/</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Medium: Fashion; thesis title 'Creating Cultural Belonging Among Immigrants Through the Lens of Kashmir'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site rupalpanwar.com, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Jiani Hu</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>jiani4942@gmail.com</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Fashion (SCAD)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://www.jianihu.com/</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Medium: Fashion; thesis title 'In Between Black and White: The Fashion Potential of Yin-Yang Philosophy in the West'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search (own site jianihu.com/resume, verified in raw HTML)</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Isaac Yu</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>isaac890302@gmail.com</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Fashion (SCAD)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://www.isaac-yu.art/</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>SCAD</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Medium: Fashion; thesis title 'Who Kills My Freedom'; from SCAD Thesis Digital Collection (library.scad.edu). Email found via Serper/Google search, corroborated on two sources (own site isaac-yu.art contact form, verified in raw HTML; also listed as 'Press Contact' on his Instagram @imisaacyu)</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:J6"/>
+  <autoFilter ref="A5:J72"/>
   <dataValidations count="2">
-    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No response,Interested,Not interested,Bounced,Follow-up needed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>